<commit_message>
Elv: ms tabela de habitat com temp e OD
</commit_message>
<xml_diff>
--- a/res/tabela de habitat.xlsx
+++ b/res/tabela de habitat.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/480d9b848b88e342/MSS/_Zoo-Rebio/ZooRebio3-23_24/rebio23-part/res/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="168" documentId="11_D9FD058DC2C30341301560FAC0A3D007D2DF5883" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AE2ABCC-8884-475A-AD21-AD84C0561592}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_210F330CE2C084B9F0295A8FC095B0388C889087" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37963647-55F6-4E5E-A1AC-CF5C5AE8FEC4}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-22425" windowWidth="21840" windowHeight="37920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20490" yWindow="-21510" windowWidth="19470" windowHeight="13380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="600">
   <si>
     <t>137.5 (119.2-164.4)</t>
   </si>
@@ -239,9 +239,6 @@
     <t>0.41 (0.33-0.557)</t>
   </si>
   <si>
-    <t>0.22 (0.115-0.37)</t>
-  </si>
-  <si>
     <t>1.4 (1-2)</t>
   </si>
   <si>
@@ -665,6 +662,228 @@
     <t>17.5 (5-25)</t>
   </si>
   <si>
+    <t>Caiana stream</t>
+  </si>
+  <si>
+    <t>Site 1</t>
+  </si>
+  <si>
+    <t>Site 2</t>
+  </si>
+  <si>
+    <t>Site 3</t>
+  </si>
+  <si>
+    <t>Site 4</t>
+  </si>
+  <si>
+    <t>Site 5</t>
+  </si>
+  <si>
+    <t>Site 6</t>
+  </si>
+  <si>
+    <t>Site 7</t>
+  </si>
+  <si>
+    <t>Site 8</t>
+  </si>
+  <si>
+    <t>Site 9</t>
+  </si>
+  <si>
+    <t>Site 10</t>
+  </si>
+  <si>
+    <t>Site 11</t>
+  </si>
+  <si>
+    <t>Site 12</t>
+  </si>
+  <si>
+    <t>Site 13</t>
+  </si>
+  <si>
+    <t>Site 14</t>
+  </si>
+  <si>
+    <t>Site 15</t>
+  </si>
+  <si>
+    <t>Conductivity (µS/cm)</t>
+  </si>
+  <si>
+    <t>Turbidity (NTU)</t>
+  </si>
+  <si>
+    <t>pH</t>
+  </si>
+  <si>
+    <t>Elevation (m a.s.l.)</t>
+  </si>
+  <si>
+    <t>Water velocity (m/s)</t>
+  </si>
+  <si>
+    <t>Slope</t>
+  </si>
+  <si>
+    <t>Average depth (cm)</t>
+  </si>
+  <si>
+    <t>Margin depth (cm)</t>
+  </si>
+  <si>
+    <t>Aquatic macrophytes</t>
+  </si>
+  <si>
+    <t>Littoral grass</t>
+  </si>
+  <si>
+    <t>Submerged vegetation</t>
+  </si>
+  <si>
+    <t>Overhanging vegetation</t>
+  </si>
+  <si>
+    <t>Leaf litter</t>
+  </si>
+  <si>
+    <t>Mud</t>
+  </si>
+  <si>
+    <t>Sand</t>
+  </si>
+  <si>
+    <t>Gravel</t>
+  </si>
+  <si>
+    <t>Rocks</t>
+  </si>
+  <si>
+    <t>Algae</t>
+  </si>
+  <si>
+    <t>Root masses</t>
+  </si>
+  <si>
+    <t>Wood debris</t>
+  </si>
+  <si>
+    <t>Water quality</t>
+  </si>
+  <si>
+    <t>Morphology</t>
+  </si>
+  <si>
+    <t>Substrate composition (%)</t>
+  </si>
+  <si>
+    <t>Habitat structures (%)</t>
+  </si>
+  <si>
+    <t>0.220 (0.115-0.37)</t>
+  </si>
+  <si>
+    <t>6.2 (3.6-14.1)</t>
+  </si>
+  <si>
+    <t>4.3 (0.7-9.2)</t>
+  </si>
+  <si>
+    <t>2 (1.1-3.2)</t>
+  </si>
+  <si>
+    <t>7.6 (2-16)</t>
+  </si>
+  <si>
+    <t>1.7 (0.8-2.5)</t>
+  </si>
+  <si>
+    <t>7.6 (4.9-10.2)</t>
+  </si>
+  <si>
+    <t>1.1 (0.2-1.9)</t>
+  </si>
+  <si>
+    <t>2 (0.9-3.7)</t>
+  </si>
+  <si>
+    <t>3.1 (1-6.7)</t>
+  </si>
+  <si>
+    <t>1.1 (0.6-1.3)</t>
+  </si>
+  <si>
+    <t>17 (8.5-26.5)</t>
+  </si>
+  <si>
+    <t>4.9 (3.4-5.8)</t>
+  </si>
+  <si>
+    <t>19.5 (5.3-34.6)</t>
+  </si>
+  <si>
+    <t>2.4 (1.4-3.3)</t>
+  </si>
+  <si>
+    <t>3.2 (2.3-5.3)</t>
+  </si>
+  <si>
+    <t>15.5 (13-17)</t>
+  </si>
+  <si>
+    <t>32.7 (27-40)</t>
+  </si>
+  <si>
+    <t>29.3 (20-47)</t>
+  </si>
+  <si>
+    <t>50.8 (35-60)</t>
+  </si>
+  <si>
+    <t>26.2 (20-34)</t>
+  </si>
+  <si>
+    <t>37.2 (20-47)</t>
+  </si>
+  <si>
+    <t>18.3 (6-36)</t>
+  </si>
+  <si>
+    <t>36.5 (13-53)</t>
+  </si>
+  <si>
+    <t>25.2 (17-45)</t>
+  </si>
+  <si>
+    <t>21.5 (14-33)</t>
+  </si>
+  <si>
+    <t>155 (110-200)</t>
+  </si>
+  <si>
+    <t>83.7 (50-110)</t>
+  </si>
+  <si>
+    <t>73.5 (28-93)</t>
+  </si>
+  <si>
+    <t>55.8 (36-79)</t>
+  </si>
+  <si>
+    <t>85.8 (55-110)</t>
+  </si>
+  <si>
+    <t>Maximum depth (cm)</t>
+  </si>
+  <si>
+    <t>Width (m)</t>
+  </si>
+  <si>
+    <t>Barro Branco stream</t>
+  </si>
+  <si>
     <t>Variable</t>
   </si>
   <si>
@@ -713,6 +932,141 @@
     <t>Ponto20</t>
   </si>
   <si>
+    <t>w.Temp.C</t>
+  </si>
+  <si>
+    <t>25.8 (24.9-27.3)</t>
+  </si>
+  <si>
+    <t>26.5 (25.3-27.5)</t>
+  </si>
+  <si>
+    <t>25.2 (24.9-25.5)</t>
+  </si>
+  <si>
+    <t>27.8 (27-28.5)</t>
+  </si>
+  <si>
+    <t>26.9 (26.6-27.3)</t>
+  </si>
+  <si>
+    <t>26.3 (26.2-26.5)</t>
+  </si>
+  <si>
+    <t>26.9 (26.5-27.4)</t>
+  </si>
+  <si>
+    <t>27.1 (27-27.2)</t>
+  </si>
+  <si>
+    <t>27.8 (27.5-28)</t>
+  </si>
+  <si>
+    <t>29.1 (29-29.3)</t>
+  </si>
+  <si>
+    <t>32.5 (31.4-33.4)</t>
+  </si>
+  <si>
+    <t>28.6 (28-29.1)</t>
+  </si>
+  <si>
+    <t>28.7 (28.5-28.9)</t>
+  </si>
+  <si>
+    <t>28.6 (28.5-28.6)</t>
+  </si>
+  <si>
+    <t>28.2 (28.1-28.2)</t>
+  </si>
+  <si>
+    <t>w.DO.mg.L</t>
+  </si>
+  <si>
+    <t>8.1 (7.8-8.5)</t>
+  </si>
+  <si>
+    <t>7.5 (7.2-7.8)</t>
+  </si>
+  <si>
+    <t>7.9 (7.7-8)</t>
+  </si>
+  <si>
+    <t>7.5 (6.5-8.4)</t>
+  </si>
+  <si>
+    <t>7.9 (7.8-7.9)</t>
+  </si>
+  <si>
+    <t>5.4 (4.9-6.1)</t>
+  </si>
+  <si>
+    <t>7.7 (6.8-8.1)</t>
+  </si>
+  <si>
+    <t>7 (6.6-7.5)</t>
+  </si>
+  <si>
+    <t>6.1 (5.1-6.8)</t>
+  </si>
+  <si>
+    <t>5.3 (5-5.4)</t>
+  </si>
+  <si>
+    <t>6.9 (6.4-7.3)</t>
+  </si>
+  <si>
+    <t>7.2 (6.1-7.8)</t>
+  </si>
+  <si>
+    <t>6.1 (5.4-7)</t>
+  </si>
+  <si>
+    <t>6.7 (6.2-7.7)</t>
+  </si>
+  <si>
+    <t>6.7 (5.2-7.7)</t>
+  </si>
+  <si>
+    <t>w.Vel.m.s</t>
+  </si>
+  <si>
+    <t>0.1 (0-0.2)</t>
+  </si>
+  <si>
+    <t>0 (0-0.1)</t>
+  </si>
+  <si>
+    <t>0.3 (0.2-0.3)</t>
+  </si>
+  <si>
+    <t>0.3 (0.1-0.6)</t>
+  </si>
+  <si>
+    <t>0.3 (0-0.4)</t>
+  </si>
+  <si>
+    <t>0.3 (0-0.5)</t>
+  </si>
+  <si>
+    <t>0.2 (0.1-0.3)</t>
+  </si>
+  <si>
+    <t>0 (0-0)</t>
+  </si>
+  <si>
+    <t>0.3 (0.1-0.5)</t>
+  </si>
+  <si>
+    <t>0.1 (0.1-0.2)</t>
+  </si>
+  <si>
+    <t>0.4 (0.3-0.6)</t>
+  </si>
+  <si>
+    <t>0.2 (0.1-0.4)</t>
+  </si>
+  <si>
     <t>w.Cond.uS.cm</t>
   </si>
   <si>
@@ -899,54 +1253,6 @@
     <t>54 (54-54)</t>
   </si>
   <si>
-    <t>m.Vel.m.s</t>
-  </si>
-  <si>
-    <t>0.073 (0.025-0.161)</t>
-  </si>
-  <si>
-    <t>0.086 (0.035-0.24)</t>
-  </si>
-  <si>
-    <t>0.135 (0.022-0.207)</t>
-  </si>
-  <si>
-    <t>0.036 (0-0.115)</t>
-  </si>
-  <si>
-    <t>0.261 (0.172-0.348)</t>
-  </si>
-  <si>
-    <t>0.04 (0-0.119)</t>
-  </si>
-  <si>
-    <t>0.271 (0.055-0.588)</t>
-  </si>
-  <si>
-    <t>0.254 (0.021-0.423)</t>
-  </si>
-  <si>
-    <t>0.296 (0.047-0.461)</t>
-  </si>
-  <si>
-    <t>0.195 (0.09-0.302)</t>
-  </si>
-  <si>
-    <t>0 (0-0)</t>
-  </si>
-  <si>
-    <t>0.272 (0.084-0.508)</t>
-  </si>
-  <si>
-    <t>0.118 (0.054-0.182)</t>
-  </si>
-  <si>
-    <t>0.41 (0.33-0.557)</t>
-  </si>
-  <si>
-    <t>0.22 (0.115-0.37)</t>
-  </si>
-  <si>
     <t>m.Slope</t>
   </si>
   <si>
@@ -1088,6 +1394,102 @@
     <t>49 (20-94)</t>
   </si>
   <si>
+    <t>m.Depth.max.cm</t>
+  </si>
+  <si>
+    <t>15.5 (13-17)</t>
+  </si>
+  <si>
+    <t>32.7 (27-40)</t>
+  </si>
+  <si>
+    <t>29.3 (20-47)</t>
+  </si>
+  <si>
+    <t>50.8 (35-60)</t>
+  </si>
+  <si>
+    <t>26.2 (20-34)</t>
+  </si>
+  <si>
+    <t>37.2 (20-47)</t>
+  </si>
+  <si>
+    <t>18.3 (6-36)</t>
+  </si>
+  <si>
+    <t>36.5 (13-53)</t>
+  </si>
+  <si>
+    <t>25.2 (17-45)</t>
+  </si>
+  <si>
+    <t>21.5 (14-33)</t>
+  </si>
+  <si>
+    <t>155 (110-200)</t>
+  </si>
+  <si>
+    <t>83.7 (50-110)</t>
+  </si>
+  <si>
+    <t>73.5 (28-93)</t>
+  </si>
+  <si>
+    <t>55.8 (36-79)</t>
+  </si>
+  <si>
+    <t>85.8 (55-110)</t>
+  </si>
+  <si>
+    <t>m.Width.m</t>
+  </si>
+  <si>
+    <t>6.2 (3.6-14.1)</t>
+  </si>
+  <si>
+    <t>4.3 (0.7-9.2)</t>
+  </si>
+  <si>
+    <t>2 (1.1-3.2)</t>
+  </si>
+  <si>
+    <t>7.6 (2-16)</t>
+  </si>
+  <si>
+    <t>1.7 (0.8-2.5)</t>
+  </si>
+  <si>
+    <t>7.6 (4.9-10.2)</t>
+  </si>
+  <si>
+    <t>1.1 (0.2-1.9)</t>
+  </si>
+  <si>
+    <t>2 (0.9-3.7)</t>
+  </si>
+  <si>
+    <t>3.1 (1-6.7)</t>
+  </si>
+  <si>
+    <t>1.1 (0.6-1.3)</t>
+  </si>
+  <si>
+    <t>17 (8.5-26.5)</t>
+  </si>
+  <si>
+    <t>4.9 (3.4-5.8)</t>
+  </si>
+  <si>
+    <t>19.5 (5.3-34.6)</t>
+  </si>
+  <si>
+    <t>2.4 (1.4-3.3)</t>
+  </si>
+  <si>
+    <t>3.2 (2.3-5.3)</t>
+  </si>
+  <si>
     <t>s.Mud</t>
   </si>
   <si>
@@ -1415,140 +1817,61 @@
     <t>17.5 (5-25)</t>
   </si>
   <si>
-    <t>Barro Branco strream</t>
-  </si>
-  <si>
-    <t>Caiana stream</t>
-  </si>
-  <si>
-    <t>Site 1</t>
-  </si>
-  <si>
-    <t>Site 2</t>
-  </si>
-  <si>
-    <t>Site 3</t>
-  </si>
-  <si>
-    <t>Site 4</t>
-  </si>
-  <si>
-    <t>Site 5</t>
-  </si>
-  <si>
-    <t>Site 6</t>
-  </si>
-  <si>
-    <t>Site 7</t>
-  </si>
-  <si>
-    <t>Site 8</t>
-  </si>
-  <si>
-    <t>Site 9</t>
-  </si>
-  <si>
-    <t>Site 10</t>
-  </si>
-  <si>
-    <t>Site 11</t>
-  </si>
-  <si>
-    <t>Site 12</t>
-  </si>
-  <si>
-    <t>Site 13</t>
-  </si>
-  <si>
-    <t>Site 14</t>
-  </si>
-  <si>
-    <t>Site 15</t>
-  </si>
-  <si>
-    <t>Conductivity (µS/cm)</t>
-  </si>
-  <si>
-    <t>Turbidity (NTU)</t>
-  </si>
-  <si>
-    <t>pH</t>
-  </si>
-  <si>
-    <t>Elevation (m a.s.l.)</t>
-  </si>
-  <si>
-    <t>Water velocity (m/s)</t>
-  </si>
-  <si>
-    <t>Slope</t>
-  </si>
-  <si>
-    <t>Average depth (cm)</t>
-  </si>
-  <si>
-    <t>Margin depth (cm)</t>
-  </si>
-  <si>
-    <t>Aquatic macrophytes</t>
-  </si>
-  <si>
-    <t>Littoral grass</t>
-  </si>
-  <si>
-    <t>Submerged vegetation</t>
-  </si>
-  <si>
-    <t>Overhanging vegetation</t>
-  </si>
-  <si>
-    <t>Leaf litter</t>
-  </si>
-  <si>
-    <t>Mud</t>
-  </si>
-  <si>
-    <t>Sand</t>
-  </si>
-  <si>
-    <t>Gravel</t>
-  </si>
-  <si>
-    <t>Rocks</t>
-  </si>
-  <si>
-    <t>Algae</t>
-  </si>
-  <si>
-    <t>Root masses</t>
-  </si>
-  <si>
-    <t>Wood debris</t>
-  </si>
-  <si>
-    <t>Water quality</t>
-  </si>
-  <si>
-    <t>Morphology</t>
-  </si>
-  <si>
-    <t>Substrate composition (%)</t>
-  </si>
-  <si>
-    <t>Habitat structures (%)</t>
+    <r>
+      <t>Temperature (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>°</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C)*</t>
+    </r>
+  </si>
+  <si>
+    <t>Dissolved oxygen (mg/L)*</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1577,18 +1900,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1604,6 +1934,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1885,1057 +2219,1257 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>214</v>
+        <v>287</v>
       </c>
       <c r="B1" t="s">
-        <v>215</v>
+        <v>288</v>
       </c>
       <c r="C1" t="s">
-        <v>216</v>
+        <v>289</v>
       </c>
       <c r="D1" t="s">
-        <v>217</v>
+        <v>290</v>
       </c>
       <c r="E1" t="s">
-        <v>218</v>
+        <v>291</v>
       </c>
       <c r="F1" t="s">
-        <v>219</v>
+        <v>292</v>
       </c>
       <c r="G1" t="s">
-        <v>220</v>
+        <v>293</v>
       </c>
       <c r="H1" t="s">
-        <v>221</v>
+        <v>294</v>
       </c>
       <c r="I1" t="s">
-        <v>222</v>
+        <v>295</v>
       </c>
       <c r="J1" t="s">
-        <v>223</v>
+        <v>296</v>
       </c>
       <c r="K1" t="s">
-        <v>224</v>
+        <v>297</v>
       </c>
       <c r="L1" t="s">
-        <v>225</v>
+        <v>298</v>
       </c>
       <c r="M1" t="s">
-        <v>226</v>
+        <v>299</v>
       </c>
       <c r="N1" t="s">
-        <v>227</v>
+        <v>300</v>
       </c>
       <c r="O1" t="s">
-        <v>228</v>
+        <v>301</v>
       </c>
       <c r="P1" t="s">
-        <v>229</v>
+        <v>302</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>230</v>
+        <v>303</v>
       </c>
       <c r="B2" t="s">
-        <v>231</v>
+        <v>304</v>
       </c>
       <c r="C2" t="s">
-        <v>232</v>
+        <v>305</v>
       </c>
       <c r="D2" t="s">
-        <v>233</v>
+        <v>306</v>
       </c>
       <c r="E2" t="s">
-        <v>234</v>
+        <v>307</v>
       </c>
       <c r="F2" t="s">
-        <v>235</v>
+        <v>308</v>
       </c>
       <c r="G2" t="s">
-        <v>236</v>
+        <v>309</v>
       </c>
       <c r="H2" t="s">
-        <v>237</v>
+        <v>310</v>
       </c>
       <c r="I2" t="s">
-        <v>238</v>
+        <v>311</v>
       </c>
       <c r="J2" t="s">
-        <v>239</v>
+        <v>312</v>
       </c>
       <c r="K2" t="s">
-        <v>240</v>
+        <v>313</v>
       </c>
       <c r="L2" t="s">
-        <v>241</v>
+        <v>314</v>
       </c>
       <c r="M2" t="s">
-        <v>242</v>
+        <v>315</v>
       </c>
       <c r="N2" t="s">
-        <v>243</v>
+        <v>316</v>
       </c>
       <c r="O2" t="s">
-        <v>244</v>
+        <v>317</v>
       </c>
       <c r="P2" t="s">
-        <v>245</v>
+        <v>318</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>246</v>
+        <v>319</v>
       </c>
       <c r="B3" t="s">
-        <v>247</v>
+        <v>320</v>
       </c>
       <c r="C3" t="s">
-        <v>248</v>
+        <v>321</v>
       </c>
       <c r="D3" t="s">
-        <v>249</v>
+        <v>322</v>
       </c>
       <c r="E3" t="s">
-        <v>250</v>
+        <v>323</v>
       </c>
       <c r="F3" t="s">
-        <v>251</v>
+        <v>324</v>
       </c>
       <c r="G3" t="s">
-        <v>252</v>
+        <v>325</v>
       </c>
       <c r="H3" t="s">
-        <v>253</v>
+        <v>326</v>
       </c>
       <c r="I3" t="s">
-        <v>254</v>
+        <v>327</v>
       </c>
       <c r="J3" t="s">
-        <v>255</v>
+        <v>328</v>
       </c>
       <c r="K3" t="s">
-        <v>256</v>
+        <v>329</v>
       </c>
       <c r="L3" t="s">
-        <v>257</v>
+        <v>330</v>
       </c>
       <c r="M3" t="s">
-        <v>258</v>
+        <v>331</v>
       </c>
       <c r="N3" t="s">
-        <v>259</v>
+        <v>332</v>
       </c>
       <c r="O3" t="s">
-        <v>260</v>
+        <v>333</v>
       </c>
       <c r="P3" t="s">
-        <v>261</v>
+        <v>334</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>262</v>
+        <v>335</v>
       </c>
       <c r="B4" t="s">
-        <v>263</v>
+        <v>336</v>
       </c>
       <c r="C4" t="s">
-        <v>264</v>
+        <v>336</v>
       </c>
       <c r="D4" t="s">
-        <v>265</v>
+        <v>336</v>
       </c>
       <c r="E4" t="s">
-        <v>266</v>
+        <v>337</v>
       </c>
       <c r="F4" t="s">
-        <v>267</v>
+        <v>338</v>
       </c>
       <c r="G4" t="s">
-        <v>268</v>
+        <v>337</v>
       </c>
       <c r="H4" t="s">
-        <v>269</v>
+        <v>339</v>
       </c>
       <c r="I4" t="s">
-        <v>270</v>
+        <v>340</v>
       </c>
       <c r="J4" t="s">
-        <v>271</v>
+        <v>341</v>
       </c>
       <c r="K4" t="s">
-        <v>272</v>
+        <v>342</v>
       </c>
       <c r="L4" t="s">
-        <v>273</v>
+        <v>343</v>
       </c>
       <c r="M4" t="s">
-        <v>274</v>
+        <v>344</v>
       </c>
       <c r="N4" t="s">
-        <v>275</v>
+        <v>345</v>
       </c>
       <c r="O4" t="s">
-        <v>276</v>
+        <v>346</v>
       </c>
       <c r="P4" t="s">
-        <v>277</v>
+        <v>347</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>278</v>
+        <v>348</v>
       </c>
       <c r="B5" t="s">
-        <v>279</v>
+        <v>349</v>
       </c>
       <c r="C5" t="s">
-        <v>280</v>
+        <v>350</v>
       </c>
       <c r="D5" t="s">
-        <v>281</v>
+        <v>351</v>
       </c>
       <c r="E5" t="s">
-        <v>282</v>
+        <v>352</v>
       </c>
       <c r="F5" t="s">
-        <v>283</v>
+        <v>353</v>
       </c>
       <c r="G5" t="s">
-        <v>284</v>
+        <v>354</v>
       </c>
       <c r="H5" t="s">
-        <v>285</v>
+        <v>355</v>
       </c>
       <c r="I5" t="s">
-        <v>286</v>
+        <v>356</v>
       </c>
       <c r="J5" t="s">
-        <v>287</v>
+        <v>357</v>
       </c>
       <c r="K5" t="s">
-        <v>288</v>
+        <v>358</v>
       </c>
       <c r="L5" t="s">
-        <v>287</v>
+        <v>359</v>
       </c>
       <c r="M5" t="s">
-        <v>289</v>
+        <v>360</v>
       </c>
       <c r="N5" t="s">
-        <v>290</v>
+        <v>361</v>
       </c>
       <c r="O5" t="s">
-        <v>291</v>
+        <v>362</v>
       </c>
       <c r="P5" t="s">
-        <v>289</v>
+        <v>363</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>292</v>
+        <v>364</v>
       </c>
       <c r="B6" t="s">
-        <v>293</v>
+        <v>365</v>
       </c>
       <c r="C6" t="s">
-        <v>294</v>
+        <v>366</v>
       </c>
       <c r="D6" t="s">
-        <v>295</v>
+        <v>367</v>
       </c>
       <c r="E6" t="s">
-        <v>296</v>
+        <v>368</v>
       </c>
       <c r="F6" t="s">
-        <v>297</v>
+        <v>369</v>
       </c>
       <c r="G6" t="s">
-        <v>298</v>
+        <v>370</v>
       </c>
       <c r="H6" t="s">
-        <v>299</v>
+        <v>371</v>
       </c>
       <c r="I6" t="s">
-        <v>300</v>
+        <v>372</v>
       </c>
       <c r="J6" t="s">
-        <v>301</v>
+        <v>373</v>
       </c>
       <c r="K6" t="s">
-        <v>302</v>
+        <v>374</v>
       </c>
       <c r="L6" t="s">
-        <v>303</v>
+        <v>375</v>
       </c>
       <c r="M6" t="s">
-        <v>304</v>
+        <v>376</v>
       </c>
       <c r="N6" t="s">
-        <v>305</v>
+        <v>377</v>
       </c>
       <c r="O6" t="s">
-        <v>306</v>
+        <v>378</v>
       </c>
       <c r="P6" t="s">
-        <v>307</v>
+        <v>379</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>308</v>
+        <v>380</v>
       </c>
       <c r="B7" t="s">
-        <v>309</v>
+        <v>381</v>
       </c>
       <c r="C7" t="s">
-        <v>310</v>
+        <v>382</v>
       </c>
       <c r="D7" t="s">
-        <v>311</v>
+        <v>383</v>
       </c>
       <c r="E7" t="s">
-        <v>312</v>
+        <v>384</v>
       </c>
       <c r="F7" t="s">
-        <v>313</v>
+        <v>385</v>
       </c>
       <c r="G7" t="s">
-        <v>314</v>
+        <v>386</v>
       </c>
       <c r="H7" t="s">
-        <v>315</v>
+        <v>387</v>
       </c>
       <c r="I7" t="s">
-        <v>316</v>
+        <v>388</v>
       </c>
       <c r="J7" t="s">
-        <v>317</v>
+        <v>389</v>
       </c>
       <c r="K7" t="s">
-        <v>318</v>
+        <v>390</v>
       </c>
       <c r="L7" t="s">
-        <v>319</v>
+        <v>391</v>
       </c>
       <c r="M7" t="s">
-        <v>320</v>
+        <v>392</v>
       </c>
       <c r="N7" t="s">
-        <v>319</v>
+        <v>393</v>
       </c>
       <c r="O7" t="s">
-        <v>321</v>
+        <v>394</v>
       </c>
       <c r="P7" t="s">
-        <v>322</v>
+        <v>395</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>323</v>
+        <v>396</v>
       </c>
       <c r="B8" t="s">
-        <v>324</v>
+        <v>397</v>
       </c>
       <c r="C8" t="s">
-        <v>325</v>
+        <v>398</v>
       </c>
       <c r="D8" t="s">
-        <v>326</v>
+        <v>399</v>
       </c>
       <c r="E8" t="s">
-        <v>327</v>
+        <v>400</v>
       </c>
       <c r="F8" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
       <c r="G8" t="s">
-        <v>329</v>
+        <v>402</v>
       </c>
       <c r="H8" t="s">
-        <v>330</v>
+        <v>403</v>
       </c>
       <c r="I8" t="s">
-        <v>331</v>
+        <v>404</v>
       </c>
       <c r="J8" t="s">
-        <v>332</v>
+        <v>405</v>
       </c>
       <c r="K8" t="s">
-        <v>333</v>
+        <v>406</v>
       </c>
       <c r="L8" t="s">
-        <v>334</v>
+        <v>405</v>
       </c>
       <c r="M8" t="s">
-        <v>335</v>
+        <v>407</v>
       </c>
       <c r="N8" t="s">
-        <v>336</v>
+        <v>408</v>
       </c>
       <c r="O8" t="s">
-        <v>337</v>
+        <v>409</v>
       </c>
       <c r="P8" t="s">
-        <v>338</v>
+        <v>407</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>339</v>
+        <v>410</v>
       </c>
       <c r="B9" t="s">
-        <v>340</v>
+        <v>411</v>
       </c>
       <c r="C9" t="s">
-        <v>341</v>
+        <v>412</v>
       </c>
       <c r="D9" t="s">
-        <v>342</v>
+        <v>413</v>
       </c>
       <c r="E9" t="s">
-        <v>343</v>
+        <v>414</v>
       </c>
       <c r="F9" t="s">
-        <v>344</v>
+        <v>415</v>
       </c>
       <c r="G9" t="s">
-        <v>345</v>
+        <v>416</v>
       </c>
       <c r="H9" t="s">
-        <v>346</v>
+        <v>417</v>
       </c>
       <c r="I9" t="s">
-        <v>347</v>
+        <v>418</v>
       </c>
       <c r="J9" t="s">
-        <v>348</v>
+        <v>419</v>
       </c>
       <c r="K9" t="s">
-        <v>349</v>
+        <v>420</v>
       </c>
       <c r="L9" t="s">
-        <v>350</v>
+        <v>421</v>
       </c>
       <c r="M9" t="s">
-        <v>351</v>
+        <v>422</v>
       </c>
       <c r="N9" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="O9" t="s">
-        <v>353</v>
+        <v>423</v>
       </c>
       <c r="P9" t="s">
-        <v>354</v>
+        <v>424</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>355</v>
+        <v>425</v>
       </c>
       <c r="B10" t="s">
-        <v>356</v>
+        <v>426</v>
       </c>
       <c r="C10" t="s">
-        <v>356</v>
+        <v>427</v>
       </c>
       <c r="D10" t="s">
-        <v>357</v>
+        <v>428</v>
       </c>
       <c r="E10" t="s">
-        <v>358</v>
+        <v>429</v>
       </c>
       <c r="F10" t="s">
-        <v>359</v>
+        <v>430</v>
       </c>
       <c r="G10" t="s">
-        <v>360</v>
+        <v>431</v>
       </c>
       <c r="H10" t="s">
-        <v>361</v>
+        <v>432</v>
       </c>
       <c r="I10" t="s">
-        <v>362</v>
+        <v>433</v>
       </c>
       <c r="J10" t="s">
-        <v>363</v>
+        <v>434</v>
       </c>
       <c r="K10" t="s">
-        <v>364</v>
+        <v>435</v>
       </c>
       <c r="L10" t="s">
-        <v>365</v>
+        <v>436</v>
       </c>
       <c r="M10" t="s">
-        <v>366</v>
+        <v>437</v>
       </c>
       <c r="N10" t="s">
-        <v>367</v>
+        <v>438</v>
       </c>
       <c r="O10" t="s">
-        <v>368</v>
+        <v>439</v>
       </c>
       <c r="P10" t="s">
-        <v>369</v>
+        <v>440</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>370</v>
+        <v>441</v>
       </c>
       <c r="B11" t="s">
-        <v>303</v>
+        <v>442</v>
       </c>
       <c r="C11" t="s">
-        <v>303</v>
+        <v>443</v>
       </c>
       <c r="D11" t="s">
-        <v>371</v>
+        <v>444</v>
       </c>
       <c r="E11" t="s">
-        <v>372</v>
+        <v>445</v>
       </c>
       <c r="F11" t="s">
-        <v>373</v>
+        <v>446</v>
       </c>
       <c r="G11" t="s">
-        <v>374</v>
+        <v>447</v>
       </c>
       <c r="H11" t="s">
-        <v>375</v>
+        <v>448</v>
       </c>
       <c r="I11" t="s">
-        <v>376</v>
+        <v>449</v>
       </c>
       <c r="J11" t="s">
-        <v>377</v>
+        <v>450</v>
       </c>
       <c r="K11" t="s">
-        <v>378</v>
+        <v>451</v>
       </c>
       <c r="L11" t="s">
-        <v>379</v>
+        <v>452</v>
       </c>
       <c r="M11" t="s">
-        <v>380</v>
+        <v>453</v>
       </c>
       <c r="N11" t="s">
-        <v>381</v>
+        <v>454</v>
       </c>
       <c r="O11" t="s">
-        <v>382</v>
+        <v>455</v>
       </c>
       <c r="P11" t="s">
-        <v>383</v>
+        <v>456</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>384</v>
+        <v>457</v>
       </c>
       <c r="B12" t="s">
-        <v>303</v>
+        <v>458</v>
       </c>
       <c r="C12" t="s">
-        <v>303</v>
+        <v>459</v>
       </c>
       <c r="D12" t="s">
-        <v>303</v>
+        <v>460</v>
       </c>
       <c r="E12" t="s">
-        <v>303</v>
+        <v>461</v>
       </c>
       <c r="F12" t="s">
-        <v>303</v>
+        <v>462</v>
       </c>
       <c r="G12" t="s">
-        <v>303</v>
+        <v>463</v>
       </c>
       <c r="H12" t="s">
-        <v>303</v>
+        <v>464</v>
       </c>
       <c r="I12" t="s">
-        <v>303</v>
+        <v>465</v>
       </c>
       <c r="J12" t="s">
-        <v>380</v>
+        <v>466</v>
       </c>
       <c r="K12" t="s">
-        <v>385</v>
+        <v>467</v>
       </c>
       <c r="L12" t="s">
-        <v>303</v>
+        <v>468</v>
       </c>
       <c r="M12" t="s">
-        <v>303</v>
+        <v>469</v>
       </c>
       <c r="N12" t="s">
-        <v>385</v>
+        <v>470</v>
       </c>
       <c r="O12" t="s">
-        <v>303</v>
+        <v>471</v>
       </c>
       <c r="P12" t="s">
-        <v>303</v>
+        <v>472</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>386</v>
+        <v>473</v>
       </c>
       <c r="B13" t="s">
-        <v>303</v>
+        <v>474</v>
       </c>
       <c r="C13" t="s">
-        <v>303</v>
+        <v>475</v>
       </c>
       <c r="D13" t="s">
-        <v>303</v>
+        <v>476</v>
       </c>
       <c r="E13" t="s">
-        <v>303</v>
+        <v>477</v>
       </c>
       <c r="F13" t="s">
-        <v>303</v>
+        <v>478</v>
       </c>
       <c r="G13" t="s">
-        <v>303</v>
+        <v>479</v>
       </c>
       <c r="H13" t="s">
-        <v>303</v>
+        <v>480</v>
       </c>
       <c r="I13" t="s">
-        <v>303</v>
+        <v>481</v>
       </c>
       <c r="J13" t="s">
-        <v>303</v>
+        <v>482</v>
       </c>
       <c r="K13" t="s">
-        <v>303</v>
+        <v>483</v>
       </c>
       <c r="L13" t="s">
-        <v>303</v>
+        <v>484</v>
       </c>
       <c r="M13" t="s">
-        <v>385</v>
+        <v>485</v>
       </c>
       <c r="N13" t="s">
-        <v>303</v>
+        <v>486</v>
       </c>
       <c r="O13" t="s">
-        <v>303</v>
+        <v>487</v>
       </c>
       <c r="P13" t="s">
-        <v>303</v>
+        <v>488</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>387</v>
+        <v>489</v>
       </c>
       <c r="B14" t="s">
-        <v>388</v>
+        <v>490</v>
       </c>
       <c r="C14" t="s">
-        <v>389</v>
+        <v>490</v>
       </c>
       <c r="D14" t="s">
-        <v>303</v>
+        <v>491</v>
       </c>
       <c r="E14" t="s">
-        <v>390</v>
+        <v>492</v>
       </c>
       <c r="F14" t="s">
-        <v>303</v>
+        <v>493</v>
       </c>
       <c r="G14" t="s">
-        <v>368</v>
+        <v>494</v>
       </c>
       <c r="H14" t="s">
-        <v>303</v>
+        <v>495</v>
       </c>
       <c r="I14" t="s">
-        <v>380</v>
+        <v>496</v>
       </c>
       <c r="J14" t="s">
-        <v>303</v>
+        <v>497</v>
       </c>
       <c r="K14" t="s">
-        <v>303</v>
+        <v>498</v>
       </c>
       <c r="L14" t="s">
-        <v>391</v>
+        <v>499</v>
       </c>
       <c r="M14" t="s">
-        <v>303</v>
+        <v>500</v>
       </c>
       <c r="N14" t="s">
-        <v>392</v>
+        <v>501</v>
       </c>
       <c r="O14" t="s">
-        <v>303</v>
+        <v>502</v>
       </c>
       <c r="P14" t="s">
-        <v>303</v>
+        <v>503</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>393</v>
+        <v>504</v>
       </c>
       <c r="B15" t="s">
-        <v>394</v>
+        <v>343</v>
       </c>
       <c r="C15" t="s">
-        <v>395</v>
+        <v>343</v>
       </c>
       <c r="D15" t="s">
-        <v>396</v>
+        <v>505</v>
       </c>
       <c r="E15" t="s">
-        <v>397</v>
+        <v>506</v>
       </c>
       <c r="F15" t="s">
-        <v>303</v>
+        <v>507</v>
       </c>
       <c r="G15" t="s">
-        <v>380</v>
+        <v>508</v>
       </c>
       <c r="H15" t="s">
-        <v>380</v>
+        <v>509</v>
       </c>
       <c r="I15" t="s">
-        <v>303</v>
+        <v>510</v>
       </c>
       <c r="J15" t="s">
-        <v>303</v>
+        <v>511</v>
       </c>
       <c r="K15" t="s">
-        <v>303</v>
+        <v>512</v>
       </c>
       <c r="L15" t="s">
-        <v>303</v>
+        <v>513</v>
       </c>
       <c r="M15" t="s">
-        <v>303</v>
+        <v>514</v>
       </c>
       <c r="N15" t="s">
-        <v>303</v>
+        <v>515</v>
       </c>
       <c r="O15" t="s">
-        <v>303</v>
+        <v>516</v>
       </c>
       <c r="P15" t="s">
-        <v>303</v>
+        <v>517</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>398</v>
+        <v>518</v>
       </c>
       <c r="B16" t="s">
-        <v>399</v>
+        <v>343</v>
       </c>
       <c r="C16" t="s">
-        <v>400</v>
+        <v>343</v>
       </c>
       <c r="D16" t="s">
-        <v>401</v>
+        <v>343</v>
       </c>
       <c r="E16" t="s">
-        <v>401</v>
+        <v>343</v>
       </c>
       <c r="F16" t="s">
-        <v>402</v>
+        <v>343</v>
       </c>
       <c r="G16" t="s">
-        <v>371</v>
+        <v>343</v>
       </c>
       <c r="H16" t="s">
-        <v>368</v>
+        <v>343</v>
       </c>
       <c r="I16" t="s">
-        <v>403</v>
+        <v>343</v>
       </c>
       <c r="J16" t="s">
-        <v>404</v>
+        <v>514</v>
       </c>
       <c r="K16" t="s">
-        <v>303</v>
+        <v>519</v>
       </c>
       <c r="L16" t="s">
-        <v>405</v>
+        <v>343</v>
       </c>
       <c r="M16" t="s">
-        <v>406</v>
+        <v>343</v>
       </c>
       <c r="N16" t="s">
-        <v>407</v>
+        <v>519</v>
       </c>
       <c r="O16" t="s">
-        <v>380</v>
+        <v>343</v>
       </c>
       <c r="P16" t="s">
-        <v>408</v>
+        <v>343</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>409</v>
+        <v>520</v>
       </c>
       <c r="B17" t="s">
-        <v>410</v>
+        <v>343</v>
       </c>
       <c r="C17" t="s">
-        <v>411</v>
+        <v>343</v>
       </c>
       <c r="D17" t="s">
-        <v>412</v>
+        <v>343</v>
       </c>
       <c r="E17" t="s">
-        <v>413</v>
+        <v>343</v>
       </c>
       <c r="F17" t="s">
-        <v>414</v>
+        <v>343</v>
       </c>
       <c r="G17" t="s">
-        <v>415</v>
+        <v>343</v>
       </c>
       <c r="H17" t="s">
-        <v>416</v>
+        <v>343</v>
       </c>
       <c r="I17" t="s">
-        <v>417</v>
+        <v>343</v>
       </c>
       <c r="J17" t="s">
-        <v>418</v>
+        <v>343</v>
       </c>
       <c r="K17" t="s">
-        <v>419</v>
+        <v>343</v>
       </c>
       <c r="L17" t="s">
-        <v>380</v>
+        <v>343</v>
       </c>
       <c r="M17" t="s">
-        <v>420</v>
+        <v>519</v>
       </c>
       <c r="N17" t="s">
-        <v>421</v>
+        <v>343</v>
       </c>
       <c r="O17" t="s">
-        <v>422</v>
+        <v>343</v>
       </c>
       <c r="P17" t="s">
-        <v>423</v>
+        <v>343</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>424</v>
+        <v>521</v>
       </c>
       <c r="B18" t="s">
-        <v>425</v>
+        <v>522</v>
       </c>
       <c r="C18" t="s">
-        <v>400</v>
+        <v>523</v>
       </c>
       <c r="D18" t="s">
-        <v>426</v>
+        <v>343</v>
       </c>
       <c r="E18" t="s">
-        <v>427</v>
+        <v>524</v>
       </c>
       <c r="F18" t="s">
-        <v>303</v>
+        <v>343</v>
       </c>
       <c r="G18" t="s">
-        <v>428</v>
+        <v>502</v>
       </c>
       <c r="H18" t="s">
-        <v>303</v>
+        <v>343</v>
       </c>
       <c r="I18" t="s">
-        <v>303</v>
+        <v>514</v>
       </c>
       <c r="J18" t="s">
-        <v>303</v>
+        <v>343</v>
       </c>
       <c r="K18" t="s">
-        <v>380</v>
+        <v>343</v>
       </c>
       <c r="L18" t="s">
-        <v>429</v>
+        <v>525</v>
       </c>
       <c r="M18" t="s">
-        <v>388</v>
+        <v>343</v>
       </c>
       <c r="N18" t="s">
-        <v>430</v>
+        <v>526</v>
       </c>
       <c r="O18" t="s">
-        <v>303</v>
+        <v>343</v>
       </c>
       <c r="P18" t="s">
-        <v>303</v>
+        <v>343</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>431</v>
+        <v>527</v>
       </c>
       <c r="B19" t="s">
-        <v>432</v>
+        <v>528</v>
       </c>
       <c r="C19" t="s">
-        <v>433</v>
+        <v>529</v>
       </c>
       <c r="D19" t="s">
-        <v>434</v>
+        <v>530</v>
       </c>
       <c r="E19" t="s">
-        <v>435</v>
+        <v>531</v>
       </c>
       <c r="F19" t="s">
-        <v>436</v>
+        <v>343</v>
       </c>
       <c r="G19" t="s">
-        <v>437</v>
+        <v>514</v>
       </c>
       <c r="H19" t="s">
-        <v>399</v>
+        <v>514</v>
       </c>
       <c r="I19" t="s">
-        <v>438</v>
+        <v>343</v>
       </c>
       <c r="J19" t="s">
-        <v>439</v>
+        <v>343</v>
       </c>
       <c r="K19" t="s">
-        <v>432</v>
+        <v>343</v>
       </c>
       <c r="L19" t="s">
-        <v>368</v>
+        <v>343</v>
       </c>
       <c r="M19" t="s">
-        <v>394</v>
+        <v>343</v>
       </c>
       <c r="N19" t="s">
-        <v>371</v>
+        <v>343</v>
       </c>
       <c r="O19" t="s">
-        <v>440</v>
+        <v>343</v>
       </c>
       <c r="P19" t="s">
-        <v>441</v>
+        <v>343</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>442</v>
+        <v>532</v>
       </c>
       <c r="B20" t="s">
-        <v>404</v>
+        <v>533</v>
       </c>
       <c r="C20" t="s">
-        <v>443</v>
+        <v>534</v>
       </c>
       <c r="D20" t="s">
-        <v>444</v>
+        <v>535</v>
       </c>
       <c r="E20" t="s">
-        <v>430</v>
+        <v>535</v>
       </c>
       <c r="F20" t="s">
-        <v>445</v>
+        <v>536</v>
       </c>
       <c r="G20" t="s">
-        <v>425</v>
+        <v>505</v>
       </c>
       <c r="H20" t="s">
-        <v>401</v>
+        <v>502</v>
       </c>
       <c r="I20" t="s">
-        <v>406</v>
+        <v>537</v>
       </c>
       <c r="J20" t="s">
-        <v>446</v>
+        <v>538</v>
       </c>
       <c r="K20" t="s">
-        <v>447</v>
+        <v>343</v>
       </c>
       <c r="L20" t="s">
-        <v>380</v>
+        <v>539</v>
       </c>
       <c r="M20" t="s">
-        <v>443</v>
+        <v>540</v>
       </c>
       <c r="N20" t="s">
-        <v>448</v>
+        <v>541</v>
       </c>
       <c r="O20" t="s">
-        <v>399</v>
+        <v>514</v>
       </c>
       <c r="P20" t="s">
-        <v>449</v>
+        <v>542</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>450</v>
+        <v>543</v>
       </c>
       <c r="B21" t="s">
-        <v>451</v>
+        <v>544</v>
       </c>
       <c r="C21" t="s">
-        <v>452</v>
+        <v>545</v>
       </c>
       <c r="D21" t="s">
-        <v>453</v>
+        <v>546</v>
       </c>
       <c r="E21" t="s">
-        <v>454</v>
+        <v>547</v>
       </c>
       <c r="F21" t="s">
-        <v>455</v>
+        <v>548</v>
       </c>
       <c r="G21" t="s">
-        <v>456</v>
+        <v>549</v>
       </c>
       <c r="H21" t="s">
-        <v>457</v>
+        <v>550</v>
       </c>
       <c r="I21" t="s">
-        <v>458</v>
+        <v>551</v>
       </c>
       <c r="J21" t="s">
-        <v>459</v>
+        <v>552</v>
       </c>
       <c r="K21" t="s">
-        <v>460</v>
+        <v>553</v>
       </c>
       <c r="L21" t="s">
-        <v>430</v>
+        <v>514</v>
       </c>
       <c r="M21" t="s">
-        <v>461</v>
+        <v>554</v>
       </c>
       <c r="N21" t="s">
-        <v>462</v>
+        <v>555</v>
       </c>
       <c r="O21" t="s">
-        <v>392</v>
+        <v>556</v>
       </c>
       <c r="P21" t="s">
-        <v>463</v>
+        <v>557</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>558</v>
+      </c>
+      <c r="B22" t="s">
+        <v>559</v>
+      </c>
+      <c r="C22" t="s">
+        <v>534</v>
+      </c>
+      <c r="D22" t="s">
+        <v>560</v>
+      </c>
+      <c r="E22" t="s">
+        <v>561</v>
+      </c>
+      <c r="F22" t="s">
+        <v>343</v>
+      </c>
+      <c r="G22" t="s">
+        <v>562</v>
+      </c>
+      <c r="H22" t="s">
+        <v>343</v>
+      </c>
+      <c r="I22" t="s">
+        <v>343</v>
+      </c>
+      <c r="J22" t="s">
+        <v>343</v>
+      </c>
+      <c r="K22" t="s">
+        <v>514</v>
+      </c>
+      <c r="L22" t="s">
+        <v>563</v>
+      </c>
+      <c r="M22" t="s">
+        <v>522</v>
+      </c>
+      <c r="N22" t="s">
+        <v>564</v>
+      </c>
+      <c r="O22" t="s">
+        <v>343</v>
+      </c>
+      <c r="P22" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>565</v>
+      </c>
+      <c r="B23" t="s">
+        <v>566</v>
+      </c>
+      <c r="C23" t="s">
+        <v>567</v>
+      </c>
+      <c r="D23" t="s">
+        <v>568</v>
+      </c>
+      <c r="E23" t="s">
+        <v>569</v>
+      </c>
+      <c r="F23" t="s">
+        <v>570</v>
+      </c>
+      <c r="G23" t="s">
+        <v>571</v>
+      </c>
+      <c r="H23" t="s">
+        <v>533</v>
+      </c>
+      <c r="I23" t="s">
+        <v>572</v>
+      </c>
+      <c r="J23" t="s">
+        <v>573</v>
+      </c>
+      <c r="K23" t="s">
+        <v>566</v>
+      </c>
+      <c r="L23" t="s">
+        <v>502</v>
+      </c>
+      <c r="M23" t="s">
+        <v>528</v>
+      </c>
+      <c r="N23" t="s">
+        <v>505</v>
+      </c>
+      <c r="O23" t="s">
+        <v>574</v>
+      </c>
+      <c r="P23" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>576</v>
+      </c>
+      <c r="B24" t="s">
+        <v>538</v>
+      </c>
+      <c r="C24" t="s">
+        <v>577</v>
+      </c>
+      <c r="D24" t="s">
+        <v>578</v>
+      </c>
+      <c r="E24" t="s">
+        <v>564</v>
+      </c>
+      <c r="F24" t="s">
+        <v>579</v>
+      </c>
+      <c r="G24" t="s">
+        <v>559</v>
+      </c>
+      <c r="H24" t="s">
+        <v>535</v>
+      </c>
+      <c r="I24" t="s">
+        <v>540</v>
+      </c>
+      <c r="J24" t="s">
+        <v>580</v>
+      </c>
+      <c r="K24" t="s">
+        <v>581</v>
+      </c>
+      <c r="L24" t="s">
+        <v>514</v>
+      </c>
+      <c r="M24" t="s">
+        <v>577</v>
+      </c>
+      <c r="N24" t="s">
+        <v>582</v>
+      </c>
+      <c r="O24" t="s">
+        <v>533</v>
+      </c>
+      <c r="P24" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>584</v>
+      </c>
+      <c r="B25" t="s">
+        <v>585</v>
+      </c>
+      <c r="C25" t="s">
+        <v>586</v>
+      </c>
+      <c r="D25" t="s">
+        <v>587</v>
+      </c>
+      <c r="E25" t="s">
+        <v>588</v>
+      </c>
+      <c r="F25" t="s">
+        <v>589</v>
+      </c>
+      <c r="G25" t="s">
+        <v>590</v>
+      </c>
+      <c r="H25" t="s">
+        <v>591</v>
+      </c>
+      <c r="I25" t="s">
+        <v>592</v>
+      </c>
+      <c r="J25" t="s">
+        <v>593</v>
+      </c>
+      <c r="K25" t="s">
+        <v>594</v>
+      </c>
+      <c r="L25" t="s">
+        <v>564</v>
+      </c>
+      <c r="M25" t="s">
+        <v>595</v>
+      </c>
+      <c r="N25" t="s">
+        <v>596</v>
+      </c>
+      <c r="O25" t="s">
+        <v>526</v>
+      </c>
+      <c r="P25" t="s">
+        <v>597</v>
       </c>
     </row>
   </sheetData>
@@ -2946,1148 +3480,1346 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B1" s="1" t="s">
-        <v>464</v>
-      </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="3" t="s">
-        <v>465</v>
-      </c>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
+      <c r="B1" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>466</v>
+        <v>214</v>
       </c>
       <c r="C2" t="s">
-        <v>467</v>
+        <v>215</v>
       </c>
       <c r="D2" t="s">
-        <v>468</v>
+        <v>216</v>
       </c>
       <c r="E2" t="s">
-        <v>469</v>
+        <v>217</v>
       </c>
       <c r="F2" t="s">
-        <v>470</v>
+        <v>218</v>
       </c>
       <c r="G2" t="s">
-        <v>471</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>472</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>473</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>474</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>475</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>476</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>478</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>479</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>480</v>
+        <v>219</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>501</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
+      <c r="A3" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>481</v>
+        <v>598</v>
       </c>
       <c r="B4" t="s">
-        <v>0</v>
+        <v>304</v>
       </c>
       <c r="C4" t="s">
-        <v>1</v>
+        <v>305</v>
       </c>
       <c r="D4" t="s">
-        <v>2</v>
+        <v>306</v>
       </c>
       <c r="E4" t="s">
-        <v>3</v>
+        <v>307</v>
       </c>
       <c r="F4" t="s">
-        <v>4</v>
+        <v>308</v>
       </c>
       <c r="G4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="M4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="N4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="O4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="P4" s="4" t="s">
-        <v>14</v>
+        <v>309</v>
+      </c>
+      <c r="H4" t="s">
+        <v>310</v>
+      </c>
+      <c r="I4" t="s">
+        <v>311</v>
+      </c>
+      <c r="J4" t="s">
+        <v>312</v>
+      </c>
+      <c r="K4" t="s">
+        <v>313</v>
+      </c>
+      <c r="L4" t="s">
+        <v>314</v>
+      </c>
+      <c r="M4" t="s">
+        <v>315</v>
+      </c>
+      <c r="N4" t="s">
+        <v>316</v>
+      </c>
+      <c r="O4" t="s">
+        <v>317</v>
+      </c>
+      <c r="P4" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>482</v>
+        <v>599</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>320</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>321</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>322</v>
       </c>
       <c r="E5" t="s">
-        <v>18</v>
+        <v>323</v>
       </c>
       <c r="F5" t="s">
-        <v>19</v>
+        <v>324</v>
       </c>
       <c r="G5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="N5" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="O5" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="P5" s="4" t="s">
-        <v>29</v>
+        <v>325</v>
+      </c>
+      <c r="H5" t="s">
+        <v>326</v>
+      </c>
+      <c r="I5" t="s">
+        <v>327</v>
+      </c>
+      <c r="J5" t="s">
+        <v>328</v>
+      </c>
+      <c r="K5" t="s">
+        <v>329</v>
+      </c>
+      <c r="L5" t="s">
+        <v>330</v>
+      </c>
+      <c r="M5" t="s">
+        <v>331</v>
+      </c>
+      <c r="N5" t="s">
+        <v>332</v>
+      </c>
+      <c r="O5" t="s">
+        <v>333</v>
+      </c>
+      <c r="P5" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>483</v>
+        <v>233</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="E6" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="F6" t="s">
-        <v>34</v>
+        <v>62</v>
       </c>
       <c r="G6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="M6" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="N6" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="O6" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="P6" s="4" t="s">
-        <v>44</v>
+        <v>63</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="L6" s="6">
+        <v>0</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>502</v>
-      </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="4"/>
-      <c r="P7" s="4"/>
+      <c r="A7" t="s">
+        <v>229</v>
+      </c>
+      <c r="B7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" t="s">
+        <v>5</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>484</v>
+        <v>230</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="E8" t="s">
-        <v>48</v>
+        <v>18</v>
       </c>
       <c r="F8" t="s">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="G8" t="s">
-        <v>50</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="L8" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="M8" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="N8" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="O8" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P8" s="4" t="s">
-        <v>55</v>
+        <v>20</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>485</v>
+        <v>231</v>
       </c>
       <c r="B9" t="s">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="E9" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="F9" t="s">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="G9" t="s">
-        <v>63</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="L9" s="4">
-        <v>0</v>
-      </c>
-      <c r="M9" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="N9" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="O9" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="P9" s="4" t="s">
-        <v>72</v>
+        <v>35</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>486</v>
-      </c>
-      <c r="B10" t="s">
-        <v>73</v>
-      </c>
-      <c r="C10" t="s">
-        <v>74</v>
-      </c>
-      <c r="D10" t="s">
-        <v>75</v>
-      </c>
-      <c r="E10" t="s">
-        <v>76</v>
-      </c>
-      <c r="F10" t="s">
-        <v>77</v>
-      </c>
-      <c r="G10" t="s">
-        <v>78</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="L10" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="M10" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="N10" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="O10" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="P10" s="4" t="s">
-        <v>86</v>
-      </c>
+      <c r="A10" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+      <c r="P10" s="1"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>487</v>
+        <v>232</v>
       </c>
       <c r="B11" t="s">
-        <v>87</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s">
-        <v>88</v>
+        <v>46</v>
       </c>
       <c r="D11" t="s">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="E11" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="F11" t="s">
-        <v>91</v>
+        <v>49</v>
       </c>
       <c r="G11" t="s">
-        <v>92</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="L11" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="M11" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="N11" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="O11" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="P11" s="4" t="s">
-        <v>101</v>
+        <v>50</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>488</v>
+        <v>234</v>
       </c>
       <c r="B12" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
       <c r="C12" t="s">
-        <v>103</v>
+        <v>73</v>
       </c>
       <c r="D12" t="s">
-        <v>104</v>
+        <v>74</v>
       </c>
       <c r="E12" t="s">
-        <v>105</v>
+        <v>75</v>
       </c>
       <c r="F12" t="s">
-        <v>106</v>
+        <v>76</v>
       </c>
       <c r="G12" t="s">
-        <v>107</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="L12" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="M12" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="N12" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="O12" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="P12" s="4" t="s">
-        <v>116</v>
+        <v>77</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>503</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
-      <c r="M13" s="4"/>
-      <c r="N13" s="4"/>
-      <c r="O13" s="4"/>
-      <c r="P13" s="4"/>
+      <c r="A13" t="s">
+        <v>235</v>
+      </c>
+      <c r="B13" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13" t="s">
+        <v>88</v>
+      </c>
+      <c r="E13" t="s">
+        <v>89</v>
+      </c>
+      <c r="F13" t="s">
+        <v>90</v>
+      </c>
+      <c r="G13" t="s">
+        <v>91</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="P13" s="1" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>494</v>
+        <v>236</v>
       </c>
       <c r="B14" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="C14" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="D14" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="E14" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="F14" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="G14" t="s">
-        <v>121</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="K14" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="L14" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="M14" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="N14" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="O14" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="P14" s="4" t="s">
-        <v>130</v>
+        <v>106</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="N14" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="P14" s="1" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>495</v>
-      </c>
-      <c r="B15">
-        <v>0</v>
-      </c>
-      <c r="C15">
-        <v>0</v>
+        <v>284</v>
+      </c>
+      <c r="B15" t="s">
+        <v>269</v>
+      </c>
+      <c r="C15" t="s">
+        <v>270</v>
       </c>
       <c r="D15" t="s">
-        <v>131</v>
+        <v>271</v>
       </c>
       <c r="E15" t="s">
-        <v>132</v>
+        <v>272</v>
       </c>
       <c r="F15" t="s">
-        <v>133</v>
+        <v>273</v>
       </c>
       <c r="G15" t="s">
-        <v>134</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="K15" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="L15" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="M15" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="N15" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="O15" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="P15" s="4" t="s">
-        <v>143</v>
+        <v>274</v>
+      </c>
+      <c r="H15" t="s">
+        <v>275</v>
+      </c>
+      <c r="I15" t="s">
+        <v>276</v>
+      </c>
+      <c r="J15" t="s">
+        <v>277</v>
+      </c>
+      <c r="K15" t="s">
+        <v>278</v>
+      </c>
+      <c r="L15" t="s">
+        <v>279</v>
+      </c>
+      <c r="M15" t="s">
+        <v>280</v>
+      </c>
+      <c r="N15" t="s">
+        <v>281</v>
+      </c>
+      <c r="O15" t="s">
+        <v>282</v>
+      </c>
+      <c r="P15" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>496</v>
-      </c>
-      <c r="B16">
-        <v>0</v>
-      </c>
-      <c r="C16">
-        <v>0</v>
-      </c>
-      <c r="D16">
-        <v>0</v>
-      </c>
-      <c r="E16">
-        <v>0</v>
-      </c>
-      <c r="F16">
-        <v>0</v>
-      </c>
-      <c r="G16">
-        <v>0</v>
-      </c>
-      <c r="H16" s="4">
-        <v>0</v>
-      </c>
-      <c r="I16" s="4">
-        <v>0</v>
-      </c>
-      <c r="J16" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="K16" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="L16" s="4">
-        <v>0</v>
-      </c>
-      <c r="M16" s="4">
-        <v>0</v>
-      </c>
-      <c r="N16" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="O16" s="4">
-        <v>0</v>
-      </c>
-      <c r="P16" s="4">
-        <v>0</v>
+        <v>285</v>
+      </c>
+      <c r="B16" t="s">
+        <v>254</v>
+      </c>
+      <c r="C16" t="s">
+        <v>255</v>
+      </c>
+      <c r="D16" t="s">
+        <v>256</v>
+      </c>
+      <c r="E16" t="s">
+        <v>257</v>
+      </c>
+      <c r="F16" t="s">
+        <v>258</v>
+      </c>
+      <c r="G16" t="s">
+        <v>259</v>
+      </c>
+      <c r="H16" t="s">
+        <v>260</v>
+      </c>
+      <c r="I16" t="s">
+        <v>261</v>
+      </c>
+      <c r="J16" t="s">
+        <v>262</v>
+      </c>
+      <c r="K16" t="s">
+        <v>263</v>
+      </c>
+      <c r="L16" t="s">
+        <v>264</v>
+      </c>
+      <c r="M16" t="s">
+        <v>265</v>
+      </c>
+      <c r="N16" t="s">
+        <v>266</v>
+      </c>
+      <c r="O16" t="s">
+        <v>267</v>
+      </c>
+      <c r="P16" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>497</v>
-      </c>
-      <c r="B17">
-        <v>0</v>
-      </c>
-      <c r="C17">
-        <v>0</v>
-      </c>
-      <c r="D17">
-        <v>0</v>
-      </c>
-      <c r="E17">
-        <v>0</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
-      <c r="G17">
-        <v>0</v>
-      </c>
-      <c r="H17" s="4">
-        <v>0</v>
-      </c>
-      <c r="I17" s="4">
-        <v>0</v>
-      </c>
-      <c r="J17" s="4">
-        <v>0</v>
-      </c>
-      <c r="K17" s="4">
-        <v>0</v>
-      </c>
-      <c r="L17" s="4">
-        <v>0</v>
-      </c>
-      <c r="M17" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="N17" s="4">
-        <v>0</v>
-      </c>
-      <c r="O17" s="4">
-        <v>0</v>
-      </c>
-      <c r="P17" s="4">
-        <v>0</v>
-      </c>
+      <c r="A17" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+      <c r="P17" s="1"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>504</v>
-      </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4"/>
-      <c r="O18" s="4"/>
-      <c r="P18" s="4"/>
+      <c r="A18" t="s">
+        <v>242</v>
+      </c>
+      <c r="B18" t="s">
+        <v>116</v>
+      </c>
+      <c r="C18" t="s">
+        <v>116</v>
+      </c>
+      <c r="D18" t="s">
+        <v>117</v>
+      </c>
+      <c r="E18" t="s">
+        <v>118</v>
+      </c>
+      <c r="F18" t="s">
+        <v>119</v>
+      </c>
+      <c r="G18" t="s">
+        <v>120</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="P18" s="1" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>489</v>
-      </c>
-      <c r="B19" t="s">
-        <v>145</v>
-      </c>
-      <c r="C19" t="s">
-        <v>146</v>
+        <v>243</v>
+      </c>
+      <c r="B19">
+        <v>0</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
       </c>
       <c r="D19" t="s">
-        <v>68</v>
+        <v>130</v>
       </c>
       <c r="E19" t="s">
-        <v>147</v>
-      </c>
-      <c r="F19">
-        <v>0</v>
+        <v>131</v>
+      </c>
+      <c r="F19" t="s">
+        <v>132</v>
       </c>
       <c r="G19" t="s">
-        <v>129</v>
-      </c>
-      <c r="H19" s="4">
-        <v>0</v>
-      </c>
-      <c r="I19" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="L19" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="M19" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="N19" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="J19" s="4">
-        <v>0</v>
-      </c>
-      <c r="K19" s="4">
-        <v>0</v>
-      </c>
-      <c r="L19" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="M19" s="4">
-        <v>0</v>
-      </c>
-      <c r="N19" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="O19" s="4">
-        <v>0</v>
-      </c>
-      <c r="P19" s="4">
-        <v>0</v>
+      <c r="O19" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="P19" s="1" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>498</v>
-      </c>
-      <c r="B20" t="s">
-        <v>188</v>
-      </c>
-      <c r="C20" t="s">
-        <v>198</v>
-      </c>
-      <c r="D20" t="s">
-        <v>199</v>
-      </c>
-      <c r="E20" t="s">
-        <v>200</v>
+        <v>244</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
       </c>
       <c r="F20">
         <v>0</v>
       </c>
-      <c r="G20" t="s">
-        <v>140</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="I20" s="4">
-        <v>0</v>
-      </c>
-      <c r="J20" s="4">
-        <v>0</v>
-      </c>
-      <c r="K20" s="4">
-        <v>0</v>
-      </c>
-      <c r="L20" s="4">
-        <v>0</v>
-      </c>
-      <c r="M20" s="4">
-        <v>0</v>
-      </c>
-      <c r="N20" s="4">
-        <v>0</v>
-      </c>
-      <c r="O20" s="4">
-        <v>0</v>
-      </c>
-      <c r="P20" s="4">
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20" s="1">
+        <v>0</v>
+      </c>
+      <c r="I20" s="1">
+        <v>0</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="L20" s="1">
+        <v>0</v>
+      </c>
+      <c r="M20" s="1">
+        <v>0</v>
+      </c>
+      <c r="N20" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="O20" s="1">
+        <v>0</v>
+      </c>
+      <c r="P20" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>491</v>
-      </c>
-      <c r="B21" t="s">
-        <v>157</v>
-      </c>
-      <c r="C21" t="s">
-        <v>151</v>
-      </c>
-      <c r="D21" t="s">
-        <v>158</v>
-      </c>
-      <c r="E21" t="s">
-        <v>158</v>
-      </c>
-      <c r="F21" t="s">
-        <v>159</v>
-      </c>
-      <c r="G21" t="s">
-        <v>131</v>
-      </c>
-      <c r="H21" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="K21" s="4">
-        <v>0</v>
-      </c>
-      <c r="L21" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="M21" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="N21" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="O21" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="P21" s="4" t="s">
-        <v>165</v>
+        <v>245</v>
+      </c>
+      <c r="B21">
+        <v>0</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21" s="1">
+        <v>0</v>
+      </c>
+      <c r="I21" s="1">
+        <v>0</v>
+      </c>
+      <c r="J21" s="1">
+        <v>0</v>
+      </c>
+      <c r="K21" s="1">
+        <v>0</v>
+      </c>
+      <c r="L21" s="1">
+        <v>0</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="N21" s="1">
+        <v>0</v>
+      </c>
+      <c r="O21" s="1">
+        <v>0</v>
+      </c>
+      <c r="P21" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>492</v>
-      </c>
-      <c r="B22" t="s">
-        <v>166</v>
-      </c>
-      <c r="C22" t="s">
-        <v>167</v>
-      </c>
-      <c r="D22" t="s">
-        <v>168</v>
-      </c>
-      <c r="E22" t="s">
-        <v>169</v>
-      </c>
-      <c r="F22" t="s">
-        <v>170</v>
-      </c>
-      <c r="G22" t="s">
-        <v>171</v>
-      </c>
-      <c r="H22" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="J22" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="K22" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="L22" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="M22" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="N22" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="O22" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="P22" s="4" t="s">
-        <v>179</v>
-      </c>
+      <c r="A22" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+      <c r="P22" s="1"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>490</v>
+        <v>237</v>
       </c>
       <c r="B23" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="C23" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="D23" t="s">
-        <v>152</v>
+        <v>68</v>
       </c>
       <c r="E23" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="F23">
         <v>0</v>
       </c>
       <c r="G23" t="s">
-        <v>154</v>
-      </c>
-      <c r="H23" s="4">
-        <v>0</v>
-      </c>
-      <c r="I23" s="4">
-        <v>0</v>
-      </c>
-      <c r="J23" s="4">
-        <v>0</v>
-      </c>
-      <c r="K23" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="L23" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="M23" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="N23" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="O23" s="4">
-        <v>0</v>
-      </c>
-      <c r="P23" s="4">
+        <v>128</v>
+      </c>
+      <c r="H23" s="1">
+        <v>0</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="J23" s="1">
+        <v>0</v>
+      </c>
+      <c r="K23" s="1">
+        <v>0</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="M23" s="1">
+        <v>0</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="O23" s="1">
+        <v>0</v>
+      </c>
+      <c r="P23" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>493</v>
+        <v>246</v>
       </c>
       <c r="B24" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="C24" t="s">
-        <v>181</v>
+        <v>197</v>
       </c>
       <c r="D24" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="E24" t="s">
-        <v>183</v>
-      </c>
-      <c r="F24" t="s">
-        <v>184</v>
+        <v>199</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
       </c>
       <c r="G24" t="s">
-        <v>185</v>
-      </c>
-      <c r="H24" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="I24" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="J24" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="K24" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="L24" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="M24" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="N24" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="O24" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="P24" s="4" t="s">
-        <v>190</v>
+        <v>139</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="I24" s="1">
+        <v>0</v>
+      </c>
+      <c r="J24" s="1">
+        <v>0</v>
+      </c>
+      <c r="K24" s="1">
+        <v>0</v>
+      </c>
+      <c r="L24" s="1">
+        <v>0</v>
+      </c>
+      <c r="M24" s="1">
+        <v>0</v>
+      </c>
+      <c r="N24" s="1">
+        <v>0</v>
+      </c>
+      <c r="O24" s="1">
+        <v>0</v>
+      </c>
+      <c r="P24" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>499</v>
+        <v>239</v>
       </c>
       <c r="B25" t="s">
+        <v>156</v>
+      </c>
+      <c r="C25" t="s">
+        <v>150</v>
+      </c>
+      <c r="D25" t="s">
+        <v>157</v>
+      </c>
+      <c r="E25" t="s">
+        <v>157</v>
+      </c>
+      <c r="F25" t="s">
+        <v>158</v>
+      </c>
+      <c r="G25" t="s">
+        <v>130</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="K25" s="1">
+        <v>0</v>
+      </c>
+      <c r="L25" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="C25" t="s">
-        <v>191</v>
-      </c>
-      <c r="D25" t="s">
-        <v>192</v>
-      </c>
-      <c r="E25" t="s">
-        <v>156</v>
-      </c>
-      <c r="F25" t="s">
-        <v>193</v>
-      </c>
-      <c r="G25" t="s">
-        <v>150</v>
-      </c>
-      <c r="H25" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="I25" s="4" t="s">
+      <c r="M25" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="N25" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="J25" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="K25" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="L25" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="M25" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="N25" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="O25" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="P25" s="4" t="s">
-        <v>197</v>
+      <c r="O25" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P25" s="1" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>500</v>
+        <v>240</v>
       </c>
       <c r="B26" t="s">
+        <v>165</v>
+      </c>
+      <c r="C26" t="s">
+        <v>166</v>
+      </c>
+      <c r="D26" t="s">
+        <v>167</v>
+      </c>
+      <c r="E26" t="s">
+        <v>168</v>
+      </c>
+      <c r="F26" t="s">
+        <v>169</v>
+      </c>
+      <c r="G26" t="s">
+        <v>170</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="L26" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="M26" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="N26" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="O26" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="P26" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>238</v>
+      </c>
+      <c r="B27" t="s">
+        <v>149</v>
+      </c>
+      <c r="C27" t="s">
+        <v>150</v>
+      </c>
+      <c r="D27" t="s">
+        <v>151</v>
+      </c>
+      <c r="E27" t="s">
+        <v>152</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27" t="s">
+        <v>153</v>
+      </c>
+      <c r="H27" s="1">
+        <v>0</v>
+      </c>
+      <c r="I27" s="1">
+        <v>0</v>
+      </c>
+      <c r="J27" s="1">
+        <v>0</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="L27" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="M27" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="N27" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="O27" s="1">
+        <v>0</v>
+      </c>
+      <c r="P27" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>241</v>
+      </c>
+      <c r="B28" t="s">
+        <v>179</v>
+      </c>
+      <c r="C28" t="s">
+        <v>180</v>
+      </c>
+      <c r="D28" t="s">
+        <v>181</v>
+      </c>
+      <c r="E28" t="s">
+        <v>182</v>
+      </c>
+      <c r="F28" t="s">
+        <v>183</v>
+      </c>
+      <c r="G28" t="s">
+        <v>184</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="L28" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="M28" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="N28" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="O28" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="P28" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>247</v>
+      </c>
+      <c r="B29" t="s">
+        <v>160</v>
+      </c>
+      <c r="C29" t="s">
+        <v>190</v>
+      </c>
+      <c r="D29" t="s">
+        <v>191</v>
+      </c>
+      <c r="E29" t="s">
+        <v>155</v>
+      </c>
+      <c r="F29" t="s">
+        <v>192</v>
+      </c>
+      <c r="G29" t="s">
+        <v>149</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="L29" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="M29" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="N29" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="O29" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="P29" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>248</v>
+      </c>
+      <c r="B30" t="s">
+        <v>200</v>
+      </c>
+      <c r="C30" t="s">
         <v>201</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D30" t="s">
         <v>202</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E30" t="s">
         <v>203</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F30" t="s">
         <v>204</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G30" t="s">
         <v>205</v>
       </c>
-      <c r="G26" t="s">
+      <c r="H30" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="I30" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="I26" s="4" t="s">
+      <c r="J30" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="J26" s="4" t="s">
+      <c r="K30" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="K26" s="4" t="s">
+      <c r="L30" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M30" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="L26" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="M26" s="4" t="s">
+      <c r="N30" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="N26" s="4" t="s">
+      <c r="O30" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="P30" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="O26" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="P26" s="4" t="s">
-        <v>213</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="B1:G1"/>
-    <mergeCell ref="H1:P1"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A7:C7"/>
+  <mergeCells count="4">
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A10:C10"/>
     <mergeCell ref="A3:C3"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Elv: ms graficos pca final
</commit_message>
<xml_diff>
--- a/res/tabela de habitat.xlsx
+++ b/res/tabela de habitat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/480d9b848b88e342/MSS/_Zoo-Rebio/ZooRebio3-23_24/rebio23-part/res/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_210F330CE2C084B9F0295A8FC095B0388C889087" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37963647-55F6-4E5E-A1AC-CF5C5AE8FEC4}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_210F330CE2C084B9F0295A8FC095B0388C889087" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{208472DD-642F-47B3-A859-E5FBC9CFA5F2}"/>
   <bookViews>
     <workbookView xWindow="-20490" yWindow="-21510" windowWidth="19470" windowHeight="13380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="600">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="599">
   <si>
     <t>137.5 (119.2-164.4)</t>
   </si>
@@ -227,9 +227,6 @@
     <t>0.195 (0.09-0.302)</t>
   </si>
   <si>
-    <t>0 (0-0)</t>
-  </si>
-  <si>
     <t>0.272 (0.084-0.508)</t>
   </si>
   <si>
@@ -768,9 +765,6 @@
   </si>
   <si>
     <t>Wood debris</t>
-  </si>
-  <si>
-    <t>Water quality</t>
   </si>
   <si>
     <t>Morphology</t>
@@ -1843,12 +1837,15 @@
   <si>
     <t>Dissolved oxygen (mg/L)*</t>
   </si>
+  <si>
+    <t>Physicochemical variables</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1872,6 +1869,13 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1900,7 +1904,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1919,6 +1923,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2224,1252 +2229,1252 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>285</v>
+      </c>
+      <c r="B1" t="s">
+        <v>286</v>
+      </c>
+      <c r="C1" t="s">
         <v>287</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>288</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>289</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>290</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>291</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>292</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>293</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>294</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>295</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>296</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>297</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>298</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>299</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
         <v>300</v>
-      </c>
-      <c r="O1" t="s">
-        <v>301</v>
-      </c>
-      <c r="P1" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B2" t="s">
+        <v>302</v>
+      </c>
+      <c r="C2" t="s">
         <v>303</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>304</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>305</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>306</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>307</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>308</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>309</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>310</v>
       </c>
-      <c r="I2" t="s">
+      <c r="K2" t="s">
         <v>311</v>
       </c>
-      <c r="J2" t="s">
+      <c r="L2" t="s">
         <v>312</v>
       </c>
-      <c r="K2" t="s">
+      <c r="M2" t="s">
         <v>313</v>
       </c>
-      <c r="L2" t="s">
+      <c r="N2" t="s">
         <v>314</v>
       </c>
-      <c r="M2" t="s">
+      <c r="O2" t="s">
         <v>315</v>
       </c>
-      <c r="N2" t="s">
+      <c r="P2" t="s">
         <v>316</v>
-      </c>
-      <c r="O2" t="s">
-        <v>317</v>
-      </c>
-      <c r="P2" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>317</v>
+      </c>
+      <c r="B3" t="s">
+        <v>318</v>
+      </c>
+      <c r="C3" t="s">
         <v>319</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>320</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>321</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>322</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>323</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>324</v>
       </c>
-      <c r="G3" t="s">
+      <c r="I3" t="s">
         <v>325</v>
       </c>
-      <c r="H3" t="s">
+      <c r="J3" t="s">
         <v>326</v>
       </c>
-      <c r="I3" t="s">
+      <c r="K3" t="s">
         <v>327</v>
       </c>
-      <c r="J3" t="s">
+      <c r="L3" t="s">
         <v>328</v>
       </c>
-      <c r="K3" t="s">
+      <c r="M3" t="s">
         <v>329</v>
       </c>
-      <c r="L3" t="s">
+      <c r="N3" t="s">
         <v>330</v>
       </c>
-      <c r="M3" t="s">
+      <c r="O3" t="s">
         <v>331</v>
       </c>
-      <c r="N3" t="s">
+      <c r="P3" t="s">
         <v>332</v>
-      </c>
-      <c r="O3" t="s">
-        <v>333</v>
-      </c>
-      <c r="P3" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>333</v>
+      </c>
+      <c r="B4" t="s">
+        <v>334</v>
+      </c>
+      <c r="C4" t="s">
+        <v>334</v>
+      </c>
+      <c r="D4" t="s">
+        <v>334</v>
+      </c>
+      <c r="E4" t="s">
         <v>335</v>
       </c>
-      <c r="B4" t="s">
+      <c r="F4" t="s">
         <v>336</v>
       </c>
-      <c r="C4" t="s">
-        <v>336</v>
-      </c>
-      <c r="D4" t="s">
-        <v>336</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="G4" t="s">
+        <v>335</v>
+      </c>
+      <c r="H4" t="s">
         <v>337</v>
       </c>
-      <c r="F4" t="s">
+      <c r="I4" t="s">
         <v>338</v>
       </c>
-      <c r="G4" t="s">
-        <v>337</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="J4" t="s">
         <v>339</v>
       </c>
-      <c r="I4" t="s">
+      <c r="K4" t="s">
         <v>340</v>
       </c>
-      <c r="J4" t="s">
-        <v>341</v>
-      </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
+        <v>341</v>
+      </c>
+      <c r="M4" t="s">
         <v>342</v>
       </c>
-      <c r="L4" t="s">
+      <c r="N4" t="s">
         <v>343</v>
       </c>
-      <c r="M4" t="s">
+      <c r="O4" t="s">
         <v>344</v>
       </c>
-      <c r="N4" t="s">
+      <c r="P4" t="s">
         <v>345</v>
-      </c>
-      <c r="O4" t="s">
-        <v>346</v>
-      </c>
-      <c r="P4" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>346</v>
+      </c>
+      <c r="B5" t="s">
+        <v>347</v>
+      </c>
+      <c r="C5" t="s">
         <v>348</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
         <v>349</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
         <v>350</v>
       </c>
-      <c r="D5" t="s">
+      <c r="F5" t="s">
         <v>351</v>
       </c>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>352</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>353</v>
       </c>
-      <c r="G5" t="s">
+      <c r="I5" t="s">
         <v>354</v>
       </c>
-      <c r="H5" t="s">
+      <c r="J5" t="s">
         <v>355</v>
       </c>
-      <c r="I5" t="s">
+      <c r="K5" t="s">
         <v>356</v>
       </c>
-      <c r="J5" t="s">
+      <c r="L5" t="s">
         <v>357</v>
       </c>
-      <c r="K5" t="s">
+      <c r="M5" t="s">
         <v>358</v>
       </c>
-      <c r="L5" t="s">
+      <c r="N5" t="s">
         <v>359</v>
       </c>
-      <c r="M5" t="s">
+      <c r="O5" t="s">
         <v>360</v>
       </c>
-      <c r="N5" t="s">
+      <c r="P5" t="s">
         <v>361</v>
-      </c>
-      <c r="O5" t="s">
-        <v>362</v>
-      </c>
-      <c r="P5" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>362</v>
+      </c>
+      <c r="B6" t="s">
+        <v>363</v>
+      </c>
+      <c r="C6" t="s">
         <v>364</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>365</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
         <v>366</v>
       </c>
-      <c r="D6" t="s">
+      <c r="F6" t="s">
         <v>367</v>
       </c>
-      <c r="E6" t="s">
+      <c r="G6" t="s">
         <v>368</v>
       </c>
-      <c r="F6" t="s">
+      <c r="H6" t="s">
         <v>369</v>
       </c>
-      <c r="G6" t="s">
+      <c r="I6" t="s">
         <v>370</v>
       </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
         <v>371</v>
       </c>
-      <c r="I6" t="s">
+      <c r="K6" t="s">
         <v>372</v>
       </c>
-      <c r="J6" t="s">
+      <c r="L6" t="s">
         <v>373</v>
       </c>
-      <c r="K6" t="s">
+      <c r="M6" t="s">
         <v>374</v>
       </c>
-      <c r="L6" t="s">
+      <c r="N6" t="s">
         <v>375</v>
       </c>
-      <c r="M6" t="s">
+      <c r="O6" t="s">
         <v>376</v>
       </c>
-      <c r="N6" t="s">
+      <c r="P6" t="s">
         <v>377</v>
-      </c>
-      <c r="O6" t="s">
-        <v>378</v>
-      </c>
-      <c r="P6" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>378</v>
+      </c>
+      <c r="B7" t="s">
+        <v>379</v>
+      </c>
+      <c r="C7" t="s">
         <v>380</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
         <v>381</v>
       </c>
-      <c r="C7" t="s">
+      <c r="E7" t="s">
         <v>382</v>
       </c>
-      <c r="D7" t="s">
+      <c r="F7" t="s">
         <v>383</v>
       </c>
-      <c r="E7" t="s">
+      <c r="G7" t="s">
         <v>384</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
         <v>385</v>
       </c>
-      <c r="G7" t="s">
+      <c r="I7" t="s">
         <v>386</v>
       </c>
-      <c r="H7" t="s">
+      <c r="J7" t="s">
         <v>387</v>
       </c>
-      <c r="I7" t="s">
+      <c r="K7" t="s">
         <v>388</v>
       </c>
-      <c r="J7" t="s">
+      <c r="L7" t="s">
         <v>389</v>
       </c>
-      <c r="K7" t="s">
+      <c r="M7" t="s">
         <v>390</v>
       </c>
-      <c r="L7" t="s">
+      <c r="N7" t="s">
         <v>391</v>
       </c>
-      <c r="M7" t="s">
+      <c r="O7" t="s">
         <v>392</v>
       </c>
-      <c r="N7" t="s">
+      <c r="P7" t="s">
         <v>393</v>
-      </c>
-      <c r="O7" t="s">
-        <v>394</v>
-      </c>
-      <c r="P7" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>394</v>
+      </c>
+      <c r="B8" t="s">
+        <v>395</v>
+      </c>
+      <c r="C8" t="s">
         <v>396</v>
       </c>
-      <c r="B8" t="s">
+      <c r="D8" t="s">
         <v>397</v>
       </c>
-      <c r="C8" t="s">
+      <c r="E8" t="s">
         <v>398</v>
       </c>
-      <c r="D8" t="s">
+      <c r="F8" t="s">
         <v>399</v>
       </c>
-      <c r="E8" t="s">
+      <c r="G8" t="s">
         <v>400</v>
       </c>
-      <c r="F8" t="s">
+      <c r="H8" t="s">
         <v>401</v>
       </c>
-      <c r="G8" t="s">
+      <c r="I8" t="s">
         <v>402</v>
       </c>
-      <c r="H8" t="s">
+      <c r="J8" t="s">
         <v>403</v>
       </c>
-      <c r="I8" t="s">
+      <c r="K8" t="s">
         <v>404</v>
       </c>
-      <c r="J8" t="s">
+      <c r="L8" t="s">
+        <v>403</v>
+      </c>
+      <c r="M8" t="s">
         <v>405</v>
       </c>
-      <c r="K8" t="s">
+      <c r="N8" t="s">
         <v>406</v>
       </c>
-      <c r="L8" t="s">
+      <c r="O8" t="s">
+        <v>407</v>
+      </c>
+      <c r="P8" t="s">
         <v>405</v>
-      </c>
-      <c r="M8" t="s">
-        <v>407</v>
-      </c>
-      <c r="N8" t="s">
-        <v>408</v>
-      </c>
-      <c r="O8" t="s">
-        <v>409</v>
-      </c>
-      <c r="P8" t="s">
-        <v>407</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>408</v>
+      </c>
+      <c r="B9" t="s">
+        <v>409</v>
+      </c>
+      <c r="C9" t="s">
         <v>410</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D9" t="s">
         <v>411</v>
       </c>
-      <c r="C9" t="s">
+      <c r="E9" t="s">
         <v>412</v>
       </c>
-      <c r="D9" t="s">
+      <c r="F9" t="s">
         <v>413</v>
       </c>
-      <c r="E9" t="s">
+      <c r="G9" t="s">
         <v>414</v>
       </c>
-      <c r="F9" t="s">
+      <c r="H9" t="s">
         <v>415</v>
       </c>
-      <c r="G9" t="s">
+      <c r="I9" t="s">
         <v>416</v>
       </c>
-      <c r="H9" t="s">
+      <c r="J9" t="s">
         <v>417</v>
       </c>
-      <c r="I9" t="s">
+      <c r="K9" t="s">
         <v>418</v>
       </c>
-      <c r="J9" t="s">
+      <c r="L9" t="s">
         <v>419</v>
       </c>
-      <c r="K9" t="s">
+      <c r="M9" t="s">
         <v>420</v>
       </c>
-      <c r="L9" t="s">
+      <c r="N9" t="s">
+        <v>419</v>
+      </c>
+      <c r="O9" t="s">
         <v>421</v>
       </c>
-      <c r="M9" t="s">
+      <c r="P9" t="s">
         <v>422</v>
-      </c>
-      <c r="N9" t="s">
-        <v>421</v>
-      </c>
-      <c r="O9" t="s">
-        <v>423</v>
-      </c>
-      <c r="P9" t="s">
-        <v>424</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>423</v>
+      </c>
+      <c r="B10" t="s">
+        <v>424</v>
+      </c>
+      <c r="C10" t="s">
         <v>425</v>
       </c>
-      <c r="B10" t="s">
+      <c r="D10" t="s">
         <v>426</v>
       </c>
-      <c r="C10" t="s">
+      <c r="E10" t="s">
         <v>427</v>
       </c>
-      <c r="D10" t="s">
+      <c r="F10" t="s">
         <v>428</v>
       </c>
-      <c r="E10" t="s">
+      <c r="G10" t="s">
         <v>429</v>
       </c>
-      <c r="F10" t="s">
+      <c r="H10" t="s">
         <v>430</v>
       </c>
-      <c r="G10" t="s">
+      <c r="I10" t="s">
         <v>431</v>
       </c>
-      <c r="H10" t="s">
+      <c r="J10" t="s">
         <v>432</v>
       </c>
-      <c r="I10" t="s">
+      <c r="K10" t="s">
         <v>433</v>
       </c>
-      <c r="J10" t="s">
+      <c r="L10" t="s">
         <v>434</v>
       </c>
-      <c r="K10" t="s">
+      <c r="M10" t="s">
         <v>435</v>
       </c>
-      <c r="L10" t="s">
+      <c r="N10" t="s">
         <v>436</v>
       </c>
-      <c r="M10" t="s">
+      <c r="O10" t="s">
         <v>437</v>
       </c>
-      <c r="N10" t="s">
+      <c r="P10" t="s">
         <v>438</v>
-      </c>
-      <c r="O10" t="s">
-        <v>439</v>
-      </c>
-      <c r="P10" t="s">
-        <v>440</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>439</v>
+      </c>
+      <c r="B11" t="s">
+        <v>440</v>
+      </c>
+      <c r="C11" t="s">
         <v>441</v>
       </c>
-      <c r="B11" t="s">
+      <c r="D11" t="s">
         <v>442</v>
       </c>
-      <c r="C11" t="s">
+      <c r="E11" t="s">
         <v>443</v>
       </c>
-      <c r="D11" t="s">
+      <c r="F11" t="s">
         <v>444</v>
       </c>
-      <c r="E11" t="s">
+      <c r="G11" t="s">
         <v>445</v>
       </c>
-      <c r="F11" t="s">
+      <c r="H11" t="s">
         <v>446</v>
       </c>
-      <c r="G11" t="s">
+      <c r="I11" t="s">
         <v>447</v>
       </c>
-      <c r="H11" t="s">
+      <c r="J11" t="s">
         <v>448</v>
       </c>
-      <c r="I11" t="s">
+      <c r="K11" t="s">
         <v>449</v>
       </c>
-      <c r="J11" t="s">
+      <c r="L11" t="s">
         <v>450</v>
       </c>
-      <c r="K11" t="s">
+      <c r="M11" t="s">
         <v>451</v>
       </c>
-      <c r="L11" t="s">
+      <c r="N11" t="s">
         <v>452</v>
       </c>
-      <c r="M11" t="s">
+      <c r="O11" t="s">
         <v>453</v>
       </c>
-      <c r="N11" t="s">
+      <c r="P11" t="s">
         <v>454</v>
-      </c>
-      <c r="O11" t="s">
-        <v>455</v>
-      </c>
-      <c r="P11" t="s">
-        <v>456</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>455</v>
+      </c>
+      <c r="B12" t="s">
+        <v>456</v>
+      </c>
+      <c r="C12" t="s">
         <v>457</v>
       </c>
-      <c r="B12" t="s">
+      <c r="D12" t="s">
         <v>458</v>
       </c>
-      <c r="C12" t="s">
+      <c r="E12" t="s">
         <v>459</v>
       </c>
-      <c r="D12" t="s">
+      <c r="F12" t="s">
         <v>460</v>
       </c>
-      <c r="E12" t="s">
+      <c r="G12" t="s">
         <v>461</v>
       </c>
-      <c r="F12" t="s">
+      <c r="H12" t="s">
         <v>462</v>
       </c>
-      <c r="G12" t="s">
+      <c r="I12" t="s">
         <v>463</v>
       </c>
-      <c r="H12" t="s">
+      <c r="J12" t="s">
         <v>464</v>
       </c>
-      <c r="I12" t="s">
+      <c r="K12" t="s">
         <v>465</v>
       </c>
-      <c r="J12" t="s">
+      <c r="L12" t="s">
         <v>466</v>
       </c>
-      <c r="K12" t="s">
+      <c r="M12" t="s">
         <v>467</v>
       </c>
-      <c r="L12" t="s">
+      <c r="N12" t="s">
         <v>468</v>
       </c>
-      <c r="M12" t="s">
+      <c r="O12" t="s">
         <v>469</v>
       </c>
-      <c r="N12" t="s">
+      <c r="P12" t="s">
         <v>470</v>
-      </c>
-      <c r="O12" t="s">
-        <v>471</v>
-      </c>
-      <c r="P12" t="s">
-        <v>472</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>471</v>
+      </c>
+      <c r="B13" t="s">
+        <v>472</v>
+      </c>
+      <c r="C13" t="s">
         <v>473</v>
       </c>
-      <c r="B13" t="s">
+      <c r="D13" t="s">
         <v>474</v>
       </c>
-      <c r="C13" t="s">
+      <c r="E13" t="s">
         <v>475</v>
       </c>
-      <c r="D13" t="s">
+      <c r="F13" t="s">
         <v>476</v>
       </c>
-      <c r="E13" t="s">
+      <c r="G13" t="s">
         <v>477</v>
       </c>
-      <c r="F13" t="s">
+      <c r="H13" t="s">
         <v>478</v>
       </c>
-      <c r="G13" t="s">
+      <c r="I13" t="s">
         <v>479</v>
       </c>
-      <c r="H13" t="s">
+      <c r="J13" t="s">
         <v>480</v>
       </c>
-      <c r="I13" t="s">
+      <c r="K13" t="s">
         <v>481</v>
       </c>
-      <c r="J13" t="s">
+      <c r="L13" t="s">
         <v>482</v>
       </c>
-      <c r="K13" t="s">
+      <c r="M13" t="s">
         <v>483</v>
       </c>
-      <c r="L13" t="s">
+      <c r="N13" t="s">
         <v>484</v>
       </c>
-      <c r="M13" t="s">
+      <c r="O13" t="s">
         <v>485</v>
       </c>
-      <c r="N13" t="s">
+      <c r="P13" t="s">
         <v>486</v>
-      </c>
-      <c r="O13" t="s">
-        <v>487</v>
-      </c>
-      <c r="P13" t="s">
-        <v>488</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>487</v>
+      </c>
+      <c r="B14" t="s">
+        <v>488</v>
+      </c>
+      <c r="C14" t="s">
+        <v>488</v>
+      </c>
+      <c r="D14" t="s">
         <v>489</v>
       </c>
-      <c r="B14" t="s">
+      <c r="E14" t="s">
         <v>490</v>
       </c>
-      <c r="C14" t="s">
-        <v>490</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="F14" t="s">
         <v>491</v>
       </c>
-      <c r="E14" t="s">
+      <c r="G14" t="s">
         <v>492</v>
       </c>
-      <c r="F14" t="s">
+      <c r="H14" t="s">
         <v>493</v>
       </c>
-      <c r="G14" t="s">
+      <c r="I14" t="s">
         <v>494</v>
       </c>
-      <c r="H14" t="s">
+      <c r="J14" t="s">
         <v>495</v>
       </c>
-      <c r="I14" t="s">
+      <c r="K14" t="s">
         <v>496</v>
       </c>
-      <c r="J14" t="s">
+      <c r="L14" t="s">
         <v>497</v>
       </c>
-      <c r="K14" t="s">
+      <c r="M14" t="s">
         <v>498</v>
       </c>
-      <c r="L14" t="s">
+      <c r="N14" t="s">
         <v>499</v>
       </c>
-      <c r="M14" t="s">
+      <c r="O14" t="s">
         <v>500</v>
       </c>
-      <c r="N14" t="s">
+      <c r="P14" t="s">
         <v>501</v>
-      </c>
-      <c r="O14" t="s">
-        <v>502</v>
-      </c>
-      <c r="P14" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>502</v>
+      </c>
+      <c r="B15" t="s">
+        <v>341</v>
+      </c>
+      <c r="C15" t="s">
+        <v>341</v>
+      </c>
+      <c r="D15" t="s">
+        <v>503</v>
+      </c>
+      <c r="E15" t="s">
         <v>504</v>
       </c>
-      <c r="B15" t="s">
-        <v>343</v>
-      </c>
-      <c r="C15" t="s">
-        <v>343</v>
-      </c>
-      <c r="D15" t="s">
+      <c r="F15" t="s">
         <v>505</v>
       </c>
-      <c r="E15" t="s">
+      <c r="G15" t="s">
         <v>506</v>
       </c>
-      <c r="F15" t="s">
+      <c r="H15" t="s">
         <v>507</v>
       </c>
-      <c r="G15" t="s">
+      <c r="I15" t="s">
         <v>508</v>
       </c>
-      <c r="H15" t="s">
+      <c r="J15" t="s">
         <v>509</v>
       </c>
-      <c r="I15" t="s">
+      <c r="K15" t="s">
         <v>510</v>
       </c>
-      <c r="J15" t="s">
+      <c r="L15" t="s">
         <v>511</v>
       </c>
-      <c r="K15" t="s">
+      <c r="M15" t="s">
         <v>512</v>
       </c>
-      <c r="L15" t="s">
+      <c r="N15" t="s">
         <v>513</v>
       </c>
-      <c r="M15" t="s">
+      <c r="O15" t="s">
         <v>514</v>
       </c>
-      <c r="N15" t="s">
+      <c r="P15" t="s">
         <v>515</v>
-      </c>
-      <c r="O15" t="s">
-        <v>516</v>
-      </c>
-      <c r="P15" t="s">
-        <v>517</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="B16" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C16" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D16" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="E16" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="F16" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="G16" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="H16" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="I16" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="J16" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="K16" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="L16" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="M16" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="N16" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="O16" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="P16" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="B17" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C17" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D17" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="E17" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="F17" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="G17" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="H17" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="I17" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="J17" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="K17" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="L17" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="M17" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="N17" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="O17" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="P17" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>519</v>
+      </c>
+      <c r="B18" t="s">
+        <v>520</v>
+      </c>
+      <c r="C18" t="s">
         <v>521</v>
       </c>
-      <c r="B18" t="s">
+      <c r="D18" t="s">
+        <v>341</v>
+      </c>
+      <c r="E18" t="s">
         <v>522</v>
       </c>
-      <c r="C18" t="s">
+      <c r="F18" t="s">
+        <v>341</v>
+      </c>
+      <c r="G18" t="s">
+        <v>500</v>
+      </c>
+      <c r="H18" t="s">
+        <v>341</v>
+      </c>
+      <c r="I18" t="s">
+        <v>512</v>
+      </c>
+      <c r="J18" t="s">
+        <v>341</v>
+      </c>
+      <c r="K18" t="s">
+        <v>341</v>
+      </c>
+      <c r="L18" t="s">
         <v>523</v>
       </c>
-      <c r="D18" t="s">
-        <v>343</v>
-      </c>
-      <c r="E18" t="s">
+      <c r="M18" t="s">
+        <v>341</v>
+      </c>
+      <c r="N18" t="s">
         <v>524</v>
       </c>
-      <c r="F18" t="s">
-        <v>343</v>
-      </c>
-      <c r="G18" t="s">
-        <v>502</v>
-      </c>
-      <c r="H18" t="s">
-        <v>343</v>
-      </c>
-      <c r="I18" t="s">
-        <v>514</v>
-      </c>
-      <c r="J18" t="s">
-        <v>343</v>
-      </c>
-      <c r="K18" t="s">
-        <v>343</v>
-      </c>
-      <c r="L18" t="s">
-        <v>525</v>
-      </c>
-      <c r="M18" t="s">
-        <v>343</v>
-      </c>
-      <c r="N18" t="s">
-        <v>526</v>
-      </c>
       <c r="O18" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="P18" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>525</v>
+      </c>
+      <c r="B19" t="s">
+        <v>526</v>
+      </c>
+      <c r="C19" t="s">
         <v>527</v>
       </c>
-      <c r="B19" t="s">
+      <c r="D19" t="s">
         <v>528</v>
       </c>
-      <c r="C19" t="s">
+      <c r="E19" t="s">
         <v>529</v>
       </c>
-      <c r="D19" t="s">
-        <v>530</v>
-      </c>
-      <c r="E19" t="s">
-        <v>531</v>
-      </c>
       <c r="F19" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="G19" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="H19" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="I19" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="J19" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="K19" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="L19" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="M19" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="N19" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="O19" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="P19" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>530</v>
+      </c>
+      <c r="B20" t="s">
+        <v>531</v>
+      </c>
+      <c r="C20" t="s">
         <v>532</v>
       </c>
-      <c r="B20" t="s">
+      <c r="D20" t="s">
         <v>533</v>
       </c>
-      <c r="C20" t="s">
+      <c r="E20" t="s">
+        <v>533</v>
+      </c>
+      <c r="F20" t="s">
         <v>534</v>
       </c>
-      <c r="D20" t="s">
+      <c r="G20" t="s">
+        <v>503</v>
+      </c>
+      <c r="H20" t="s">
+        <v>500</v>
+      </c>
+      <c r="I20" t="s">
         <v>535</v>
       </c>
-      <c r="E20" t="s">
-        <v>535</v>
-      </c>
-      <c r="F20" t="s">
+      <c r="J20" t="s">
         <v>536</v>
       </c>
-      <c r="G20" t="s">
-        <v>505</v>
-      </c>
-      <c r="H20" t="s">
-        <v>502</v>
-      </c>
-      <c r="I20" t="s">
+      <c r="K20" t="s">
+        <v>341</v>
+      </c>
+      <c r="L20" t="s">
         <v>537</v>
       </c>
-      <c r="J20" t="s">
+      <c r="M20" t="s">
         <v>538</v>
       </c>
-      <c r="K20" t="s">
-        <v>343</v>
-      </c>
-      <c r="L20" t="s">
+      <c r="N20" t="s">
         <v>539</v>
       </c>
-      <c r="M20" t="s">
+      <c r="O20" t="s">
+        <v>512</v>
+      </c>
+      <c r="P20" t="s">
         <v>540</v>
-      </c>
-      <c r="N20" t="s">
-        <v>541</v>
-      </c>
-      <c r="O20" t="s">
-        <v>514</v>
-      </c>
-      <c r="P20" t="s">
-        <v>542</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>541</v>
+      </c>
+      <c r="B21" t="s">
+        <v>542</v>
+      </c>
+      <c r="C21" t="s">
         <v>543</v>
       </c>
-      <c r="B21" t="s">
+      <c r="D21" t="s">
         <v>544</v>
       </c>
-      <c r="C21" t="s">
+      <c r="E21" t="s">
         <v>545</v>
       </c>
-      <c r="D21" t="s">
+      <c r="F21" t="s">
         <v>546</v>
       </c>
-      <c r="E21" t="s">
+      <c r="G21" t="s">
         <v>547</v>
       </c>
-      <c r="F21" t="s">
+      <c r="H21" t="s">
         <v>548</v>
       </c>
-      <c r="G21" t="s">
+      <c r="I21" t="s">
         <v>549</v>
       </c>
-      <c r="H21" t="s">
+      <c r="J21" t="s">
         <v>550</v>
       </c>
-      <c r="I21" t="s">
+      <c r="K21" t="s">
         <v>551</v>
       </c>
-      <c r="J21" t="s">
+      <c r="L21" t="s">
+        <v>512</v>
+      </c>
+      <c r="M21" t="s">
         <v>552</v>
       </c>
-      <c r="K21" t="s">
+      <c r="N21" t="s">
         <v>553</v>
       </c>
-      <c r="L21" t="s">
-        <v>514</v>
-      </c>
-      <c r="M21" t="s">
+      <c r="O21" t="s">
         <v>554</v>
       </c>
-      <c r="N21" t="s">
+      <c r="P21" t="s">
         <v>555</v>
-      </c>
-      <c r="O21" t="s">
-        <v>556</v>
-      </c>
-      <c r="P21" t="s">
-        <v>557</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>556</v>
+      </c>
+      <c r="B22" t="s">
+        <v>557</v>
+      </c>
+      <c r="C22" t="s">
+        <v>532</v>
+      </c>
+      <c r="D22" t="s">
         <v>558</v>
       </c>
-      <c r="B22" t="s">
+      <c r="E22" t="s">
         <v>559</v>
       </c>
-      <c r="C22" t="s">
-        <v>534</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="F22" t="s">
+        <v>341</v>
+      </c>
+      <c r="G22" t="s">
         <v>560</v>
       </c>
-      <c r="E22" t="s">
+      <c r="H22" t="s">
+        <v>341</v>
+      </c>
+      <c r="I22" t="s">
+        <v>341</v>
+      </c>
+      <c r="J22" t="s">
+        <v>341</v>
+      </c>
+      <c r="K22" t="s">
+        <v>512</v>
+      </c>
+      <c r="L22" t="s">
         <v>561</v>
       </c>
-      <c r="F22" t="s">
-        <v>343</v>
-      </c>
-      <c r="G22" t="s">
+      <c r="M22" t="s">
+        <v>520</v>
+      </c>
+      <c r="N22" t="s">
         <v>562</v>
       </c>
-      <c r="H22" t="s">
-        <v>343</v>
-      </c>
-      <c r="I22" t="s">
-        <v>343</v>
-      </c>
-      <c r="J22" t="s">
-        <v>343</v>
-      </c>
-      <c r="K22" t="s">
-        <v>514</v>
-      </c>
-      <c r="L22" t="s">
-        <v>563</v>
-      </c>
-      <c r="M22" t="s">
-        <v>522</v>
-      </c>
-      <c r="N22" t="s">
-        <v>564</v>
-      </c>
       <c r="O22" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="P22" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>563</v>
+      </c>
+      <c r="B23" t="s">
+        <v>564</v>
+      </c>
+      <c r="C23" t="s">
         <v>565</v>
       </c>
-      <c r="B23" t="s">
+      <c r="D23" t="s">
         <v>566</v>
       </c>
-      <c r="C23" t="s">
+      <c r="E23" t="s">
         <v>567</v>
       </c>
-      <c r="D23" t="s">
+      <c r="F23" t="s">
         <v>568</v>
       </c>
-      <c r="E23" t="s">
+      <c r="G23" t="s">
         <v>569</v>
       </c>
-      <c r="F23" t="s">
+      <c r="H23" t="s">
+        <v>531</v>
+      </c>
+      <c r="I23" t="s">
         <v>570</v>
       </c>
-      <c r="G23" t="s">
+      <c r="J23" t="s">
         <v>571</v>
       </c>
-      <c r="H23" t="s">
-        <v>533</v>
-      </c>
-      <c r="I23" t="s">
+      <c r="K23" t="s">
+        <v>564</v>
+      </c>
+      <c r="L23" t="s">
+        <v>500</v>
+      </c>
+      <c r="M23" t="s">
+        <v>526</v>
+      </c>
+      <c r="N23" t="s">
+        <v>503</v>
+      </c>
+      <c r="O23" t="s">
         <v>572</v>
       </c>
-      <c r="J23" t="s">
+      <c r="P23" t="s">
         <v>573</v>
-      </c>
-      <c r="K23" t="s">
-        <v>566</v>
-      </c>
-      <c r="L23" t="s">
-        <v>502</v>
-      </c>
-      <c r="M23" t="s">
-        <v>528</v>
-      </c>
-      <c r="N23" t="s">
-        <v>505</v>
-      </c>
-      <c r="O23" t="s">
-        <v>574</v>
-      </c>
-      <c r="P23" t="s">
-        <v>575</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>574</v>
+      </c>
+      <c r="B24" t="s">
+        <v>536</v>
+      </c>
+      <c r="C24" t="s">
+        <v>575</v>
+      </c>
+      <c r="D24" t="s">
         <v>576</v>
       </c>
-      <c r="B24" t="s">
+      <c r="E24" t="s">
+        <v>562</v>
+      </c>
+      <c r="F24" t="s">
+        <v>577</v>
+      </c>
+      <c r="G24" t="s">
+        <v>557</v>
+      </c>
+      <c r="H24" t="s">
+        <v>533</v>
+      </c>
+      <c r="I24" t="s">
         <v>538</v>
       </c>
-      <c r="C24" t="s">
-        <v>577</v>
-      </c>
-      <c r="D24" t="s">
+      <c r="J24" t="s">
         <v>578</v>
       </c>
-      <c r="E24" t="s">
-        <v>564</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="K24" t="s">
         <v>579</v>
       </c>
-      <c r="G24" t="s">
-        <v>559</v>
-      </c>
-      <c r="H24" t="s">
-        <v>535</v>
-      </c>
-      <c r="I24" t="s">
-        <v>540</v>
-      </c>
-      <c r="J24" t="s">
+      <c r="L24" t="s">
+        <v>512</v>
+      </c>
+      <c r="M24" t="s">
+        <v>575</v>
+      </c>
+      <c r="N24" t="s">
         <v>580</v>
       </c>
-      <c r="K24" t="s">
+      <c r="O24" t="s">
+        <v>531</v>
+      </c>
+      <c r="P24" t="s">
         <v>581</v>
-      </c>
-      <c r="L24" t="s">
-        <v>514</v>
-      </c>
-      <c r="M24" t="s">
-        <v>577</v>
-      </c>
-      <c r="N24" t="s">
-        <v>582</v>
-      </c>
-      <c r="O24" t="s">
-        <v>533</v>
-      </c>
-      <c r="P24" t="s">
-        <v>583</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>582</v>
+      </c>
+      <c r="B25" t="s">
+        <v>583</v>
+      </c>
+      <c r="C25" t="s">
         <v>584</v>
       </c>
-      <c r="B25" t="s">
+      <c r="D25" t="s">
         <v>585</v>
       </c>
-      <c r="C25" t="s">
+      <c r="E25" t="s">
         <v>586</v>
       </c>
-      <c r="D25" t="s">
+      <c r="F25" t="s">
         <v>587</v>
       </c>
-      <c r="E25" t="s">
+      <c r="G25" t="s">
         <v>588</v>
       </c>
-      <c r="F25" t="s">
+      <c r="H25" t="s">
         <v>589</v>
       </c>
-      <c r="G25" t="s">
+      <c r="I25" t="s">
         <v>590</v>
       </c>
-      <c r="H25" t="s">
+      <c r="J25" t="s">
         <v>591</v>
       </c>
-      <c r="I25" t="s">
+      <c r="K25" t="s">
         <v>592</v>
       </c>
-      <c r="J25" t="s">
+      <c r="L25" t="s">
+        <v>562</v>
+      </c>
+      <c r="M25" t="s">
         <v>593</v>
       </c>
-      <c r="K25" t="s">
+      <c r="N25" t="s">
         <v>594</v>
       </c>
-      <c r="L25" t="s">
-        <v>564</v>
-      </c>
-      <c r="M25" t="s">
+      <c r="O25" t="s">
+        <v>524</v>
+      </c>
+      <c r="P25" t="s">
         <v>595</v>
-      </c>
-      <c r="N25" t="s">
-        <v>596</v>
-      </c>
-      <c r="O25" t="s">
-        <v>526</v>
-      </c>
-      <c r="P25" t="s">
-        <v>597</v>
       </c>
     </row>
   </sheetData>
@@ -3485,7 +3490,7 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -3493,7 +3498,7 @@
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
       <c r="H1" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
@@ -3506,54 +3511,54 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C2" t="s">
         <v>214</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>215</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>216</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>217</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>218</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>227</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>249</v>
+        <v>598</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -3569,107 +3574,107 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="B4" t="s">
+        <v>302</v>
+      </c>
+      <c r="C4" t="s">
+        <v>303</v>
+      </c>
+      <c r="D4" t="s">
         <v>304</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
         <v>305</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
         <v>306</v>
       </c>
-      <c r="E4" t="s">
+      <c r="G4" t="s">
         <v>307</v>
       </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>308</v>
       </c>
-      <c r="G4" t="s">
+      <c r="I4" t="s">
         <v>309</v>
       </c>
-      <c r="H4" t="s">
+      <c r="J4" t="s">
         <v>310</v>
       </c>
-      <c r="I4" t="s">
+      <c r="K4" t="s">
         <v>311</v>
       </c>
-      <c r="J4" t="s">
+      <c r="L4" t="s">
         <v>312</v>
       </c>
-      <c r="K4" t="s">
+      <c r="M4" t="s">
         <v>313</v>
       </c>
-      <c r="L4" t="s">
+      <c r="N4" t="s">
         <v>314</v>
       </c>
-      <c r="M4" t="s">
+      <c r="O4" t="s">
         <v>315</v>
       </c>
-      <c r="N4" t="s">
+      <c r="P4" t="s">
         <v>316</v>
-      </c>
-      <c r="O4" t="s">
-        <v>317</v>
-      </c>
-      <c r="P4" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="B5" t="s">
+        <v>318</v>
+      </c>
+      <c r="C5" t="s">
+        <v>319</v>
+      </c>
+      <c r="D5" t="s">
         <v>320</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
         <v>321</v>
       </c>
-      <c r="D5" t="s">
+      <c r="F5" t="s">
         <v>322</v>
       </c>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>323</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>324</v>
       </c>
-      <c r="G5" t="s">
+      <c r="I5" t="s">
         <v>325</v>
       </c>
-      <c r="H5" t="s">
+      <c r="J5" t="s">
         <v>326</v>
       </c>
-      <c r="I5" t="s">
+      <c r="K5" t="s">
         <v>327</v>
       </c>
-      <c r="J5" t="s">
+      <c r="L5" t="s">
         <v>328</v>
       </c>
-      <c r="K5" t="s">
+      <c r="M5" t="s">
         <v>329</v>
       </c>
-      <c r="L5" t="s">
+      <c r="N5" t="s">
         <v>330</v>
       </c>
-      <c r="M5" t="s">
+      <c r="O5" t="s">
         <v>331</v>
       </c>
-      <c r="N5" t="s">
+      <c r="P5" t="s">
         <v>332</v>
-      </c>
-      <c r="O5" t="s">
-        <v>333</v>
-      </c>
-      <c r="P5" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B6" t="s">
         <v>58</v>
@@ -3705,21 +3710,21 @@
         <v>0</v>
       </c>
       <c r="M6" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="N6" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="N6" s="1" t="s">
+      <c r="O6" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="O6" s="6" t="s">
-        <v>71</v>
-      </c>
       <c r="P6" s="1" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B7" t="s">
         <v>0</v>
@@ -3769,7 +3774,7 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
@@ -3819,7 +3824,7 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B9" t="s">
         <v>30</v>
@@ -3869,7 +3874,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
@@ -3885,7 +3890,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B11" t="s">
         <v>45</v>
@@ -3935,257 +3940,257 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C12" t="s">
         <v>72</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>73</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>74</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>75</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>76</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="I12" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="J12" s="1" t="s">
+      <c r="K12" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="K12" s="1" t="s">
+      <c r="L12" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L12" s="1" t="s">
+      <c r="M12" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="M12" s="1" t="s">
+      <c r="N12" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O12" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N12" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="O12" s="1" t="s">
+      <c r="P12" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="P12" s="1" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" t="s">
         <v>86</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>87</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>88</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>89</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>90</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="I13" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="K13" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="L13" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="L13" s="1" t="s">
+      <c r="M13" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="M13" s="1" t="s">
+      <c r="N13" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="N13" s="1" t="s">
+      <c r="O13" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="O13" s="1" t="s">
+      <c r="P13" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="P13" s="1" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B14" t="s">
+        <v>100</v>
+      </c>
+      <c r="C14" t="s">
         <v>101</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>102</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>103</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>104</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>105</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="I14" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="K14" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="L14" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="L14" s="1" t="s">
+      <c r="M14" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="M14" s="1" t="s">
+      <c r="N14" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="N14" s="1" t="s">
+      <c r="O14" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="O14" s="1" t="s">
+      <c r="P14" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="P14" s="1" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B15" t="s">
+        <v>267</v>
+      </c>
+      <c r="C15" t="s">
+        <v>268</v>
+      </c>
+      <c r="D15" t="s">
         <v>269</v>
       </c>
-      <c r="C15" t="s">
+      <c r="E15" t="s">
         <v>270</v>
       </c>
-      <c r="D15" t="s">
+      <c r="F15" t="s">
         <v>271</v>
       </c>
-      <c r="E15" t="s">
+      <c r="G15" t="s">
         <v>272</v>
       </c>
-      <c r="F15" t="s">
+      <c r="H15" t="s">
         <v>273</v>
       </c>
-      <c r="G15" t="s">
+      <c r="I15" t="s">
         <v>274</v>
       </c>
-      <c r="H15" t="s">
+      <c r="J15" t="s">
         <v>275</v>
       </c>
-      <c r="I15" t="s">
+      <c r="K15" t="s">
         <v>276</v>
       </c>
-      <c r="J15" t="s">
+      <c r="L15" t="s">
         <v>277</v>
       </c>
-      <c r="K15" t="s">
+      <c r="M15" t="s">
         <v>278</v>
       </c>
-      <c r="L15" t="s">
+      <c r="N15" t="s">
         <v>279</v>
       </c>
-      <c r="M15" t="s">
+      <c r="O15" t="s">
         <v>280</v>
       </c>
-      <c r="N15" t="s">
+      <c r="P15" t="s">
         <v>281</v>
-      </c>
-      <c r="O15" t="s">
-        <v>282</v>
-      </c>
-      <c r="P15" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B16" t="s">
+        <v>252</v>
+      </c>
+      <c r="C16" t="s">
+        <v>253</v>
+      </c>
+      <c r="D16" t="s">
         <v>254</v>
       </c>
-      <c r="C16" t="s">
+      <c r="E16" t="s">
         <v>255</v>
       </c>
-      <c r="D16" t="s">
+      <c r="F16" t="s">
         <v>256</v>
       </c>
-      <c r="E16" t="s">
+      <c r="G16" t="s">
         <v>257</v>
       </c>
-      <c r="F16" t="s">
+      <c r="H16" t="s">
         <v>258</v>
       </c>
-      <c r="G16" t="s">
+      <c r="I16" t="s">
         <v>259</v>
       </c>
-      <c r="H16" t="s">
+      <c r="J16" t="s">
         <v>260</v>
       </c>
-      <c r="I16" t="s">
+      <c r="K16" t="s">
         <v>261</v>
       </c>
-      <c r="J16" t="s">
+      <c r="L16" t="s">
         <v>262</v>
       </c>
-      <c r="K16" t="s">
+      <c r="M16" t="s">
         <v>263</v>
       </c>
-      <c r="L16" t="s">
+      <c r="N16" t="s">
         <v>264</v>
       </c>
-      <c r="M16" t="s">
+      <c r="O16" t="s">
         <v>265</v>
       </c>
-      <c r="N16" t="s">
+      <c r="P16" t="s">
         <v>266</v>
-      </c>
-      <c r="O16" t="s">
-        <v>267</v>
-      </c>
-      <c r="P16" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -4201,57 +4206,57 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>242</v>
-      </c>
-      <c r="B18" t="s">
+        <v>241</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D18" t="s">
         <v>116</v>
       </c>
-      <c r="C18" t="s">
-        <v>116</v>
-      </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>117</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>118</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>119</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="I18" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="J18" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="J18" s="1" t="s">
+      <c r="K18" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="L18" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="L18" s="1" t="s">
+      <c r="M18" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="M18" s="1" t="s">
+      <c r="N18" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="N18" s="1" t="s">
+      <c r="O18" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="O18" s="1" t="s">
+      <c r="P18" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="P18" s="1" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -4260,48 +4265,48 @@
         <v>0</v>
       </c>
       <c r="D19" t="s">
+        <v>129</v>
+      </c>
+      <c r="E19" t="s">
         <v>130</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>131</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>132</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="H19" s="1" t="s">
+      <c r="I19" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="I19" s="1" t="s">
+      <c r="J19" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="J19" s="1" t="s">
+      <c r="K19" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="K19" s="1" t="s">
+      <c r="L19" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="L19" s="1" t="s">
+      <c r="M19" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="M19" s="1" t="s">
+      <c r="N19" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="N19" s="1" t="s">
+      <c r="O19" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="O19" s="1" t="s">
+      <c r="P19" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="P19" s="1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -4328,10 +4333,10 @@
         <v>0</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L20" s="1">
         <v>0</v>
@@ -4340,7 +4345,7 @@
         <v>0</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O20" s="1">
         <v>0</v>
@@ -4351,7 +4356,7 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -4387,7 +4392,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="N21" s="1">
         <v>0</v>
@@ -4401,7 +4406,7 @@
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -4417,402 +4422,402 @@
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B23" t="s">
+        <v>143</v>
+      </c>
+      <c r="C23" t="s">
         <v>144</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" s="8">
+        <v>0</v>
+      </c>
+      <c r="E23" t="s">
         <v>145</v>
       </c>
-      <c r="D23" t="s">
-        <v>68</v>
-      </c>
-      <c r="E23" t="s">
+      <c r="F23" s="8">
+        <v>0</v>
+      </c>
+      <c r="G23" t="s">
+        <v>127</v>
+      </c>
+      <c r="H23" s="6">
+        <v>0</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="J23" s="6">
+        <v>0</v>
+      </c>
+      <c r="K23" s="1">
+        <v>0</v>
+      </c>
+      <c r="L23" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="F23">
-        <v>0</v>
-      </c>
-      <c r="G23" t="s">
-        <v>128</v>
-      </c>
-      <c r="H23" s="1">
-        <v>0</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="J23" s="1">
-        <v>0</v>
-      </c>
-      <c r="K23" s="1">
-        <v>0</v>
-      </c>
-      <c r="L23" s="1" t="s">
+      <c r="M23" s="1">
+        <v>0</v>
+      </c>
+      <c r="N23" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="M23" s="1">
-        <v>0</v>
-      </c>
-      <c r="N23" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="O23" s="1">
-        <v>0</v>
-      </c>
-      <c r="P23" s="1">
+      <c r="O23" s="6">
+        <v>0</v>
+      </c>
+      <c r="P23" s="6">
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B24" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C24" t="s">
+        <v>196</v>
+      </c>
+      <c r="D24" t="s">
         <v>197</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>198</v>
       </c>
-      <c r="E24" t="s">
-        <v>199</v>
-      </c>
-      <c r="F24">
+      <c r="F24" s="8">
         <v>0</v>
       </c>
       <c r="G24" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="I24" s="1">
-        <v>0</v>
-      </c>
-      <c r="J24" s="1">
-        <v>0</v>
-      </c>
-      <c r="K24" s="1">
-        <v>0</v>
-      </c>
-      <c r="L24" s="1">
-        <v>0</v>
-      </c>
-      <c r="M24" s="1">
-        <v>0</v>
-      </c>
-      <c r="N24" s="1">
-        <v>0</v>
-      </c>
-      <c r="O24" s="1">
-        <v>0</v>
-      </c>
-      <c r="P24" s="1">
+        <v>138</v>
+      </c>
+      <c r="I24" s="6">
+        <v>0</v>
+      </c>
+      <c r="J24" s="6">
+        <v>0</v>
+      </c>
+      <c r="K24" s="6">
+        <v>0</v>
+      </c>
+      <c r="L24" s="6">
+        <v>0</v>
+      </c>
+      <c r="M24" s="6">
+        <v>0</v>
+      </c>
+      <c r="N24" s="6">
+        <v>0</v>
+      </c>
+      <c r="O24" s="6">
+        <v>0</v>
+      </c>
+      <c r="P24" s="6">
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B25" t="s">
+        <v>155</v>
+      </c>
+      <c r="C25" t="s">
+        <v>149</v>
+      </c>
+      <c r="D25" t="s">
         <v>156</v>
       </c>
-      <c r="C25" t="s">
-        <v>150</v>
-      </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
+        <v>156</v>
+      </c>
+      <c r="F25" t="s">
         <v>157</v>
       </c>
-      <c r="E25" t="s">
-        <v>157</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
+        <v>129</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="I25" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="G25" t="s">
-        <v>130</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="I25" s="1" t="s">
+      <c r="J25" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="J25" s="1" t="s">
+      <c r="K25" s="1">
+        <v>0</v>
+      </c>
+      <c r="L25" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="K25" s="1">
-        <v>0</v>
-      </c>
-      <c r="L25" s="1" t="s">
+      <c r="M25" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="M25" s="1" t="s">
+      <c r="N25" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="N25" s="1" t="s">
+      <c r="O25" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="P25" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="O25" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="P25" s="1" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B26" t="s">
+        <v>164</v>
+      </c>
+      <c r="C26" t="s">
         <v>165</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>166</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>167</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>168</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>169</v>
       </c>
-      <c r="G26" t="s">
+      <c r="H26" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="I26" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I26" s="1" t="s">
+      <c r="J26" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="J26" s="1" t="s">
+      <c r="K26" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="K26" s="1" t="s">
+      <c r="L26" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="M26" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L26" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="M26" s="1" t="s">
+      <c r="N26" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="N26" s="1" t="s">
+      <c r="O26" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="O26" s="1" t="s">
+      <c r="P26" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="P26" s="1" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B27" t="s">
+        <v>148</v>
+      </c>
+      <c r="C27" t="s">
         <v>149</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>150</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>151</v>
       </c>
-      <c r="E27" t="s">
+      <c r="F27" s="8">
+        <v>0</v>
+      </c>
+      <c r="G27" t="s">
         <v>152</v>
       </c>
-      <c r="F27">
-        <v>0</v>
-      </c>
-      <c r="G27" t="s">
+      <c r="H27" s="6">
+        <v>0</v>
+      </c>
+      <c r="I27" s="6">
+        <v>0</v>
+      </c>
+      <c r="J27" s="6">
+        <v>0</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="L27" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="H27" s="1">
-        <v>0</v>
-      </c>
-      <c r="I27" s="1">
-        <v>0</v>
-      </c>
-      <c r="J27" s="1">
-        <v>0</v>
-      </c>
-      <c r="K27" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="L27" s="1" t="s">
+      <c r="M27" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="N27" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="M27" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="N27" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="O27" s="1">
-        <v>0</v>
-      </c>
-      <c r="P27" s="1">
+      <c r="O27" s="6">
+        <v>0</v>
+      </c>
+      <c r="P27" s="6">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B28" t="s">
+        <v>178</v>
+      </c>
+      <c r="C28" t="s">
         <v>179</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>180</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>181</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
         <v>182</v>
       </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
         <v>183</v>
       </c>
-      <c r="G28" t="s">
+      <c r="H28" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="I28" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="H28" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="I28" s="1" t="s">
+      <c r="J28" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="J28" s="1" t="s">
+      <c r="K28" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="L28" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="M28" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="K28" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="L28" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="M28" s="1" t="s">
+      <c r="N28" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="O28" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="N28" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="O28" s="1" t="s">
+      <c r="P28" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="P28" s="1" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B29" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C29" t="s">
+        <v>189</v>
+      </c>
+      <c r="D29" t="s">
         <v>190</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
+        <v>154</v>
+      </c>
+      <c r="F29" t="s">
         <v>191</v>
       </c>
-      <c r="E29" t="s">
+      <c r="G29" t="s">
+        <v>148</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="L29" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="M29" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="N29" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="O29" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="F29" t="s">
-        <v>192</v>
-      </c>
-      <c r="G29" t="s">
-        <v>149</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="K29" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="L29" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="M29" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="N29" s="1" t="s">
+      <c r="P29" s="1" t="s">
         <v>195</v>
-      </c>
-      <c r="O29" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="P29" s="1" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B30" t="s">
+        <v>199</v>
+      </c>
+      <c r="C30" t="s">
         <v>200</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>201</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>202</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
         <v>203</v>
       </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
         <v>204</v>
       </c>
-      <c r="G30" t="s">
+      <c r="H30" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="I30" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="I30" s="1" t="s">
+      <c r="J30" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="J30" s="1" t="s">
+      <c r="K30" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="K30" s="1" t="s">
+      <c r="L30" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="M30" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="L30" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="M30" s="1" t="s">
+      <c r="N30" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="N30" s="1" t="s">
+      <c r="O30" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="P30" s="1" t="s">
         <v>211</v>
-      </c>
-      <c r="O30" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="P30" s="1" t="s">
-        <v>212</v>
       </c>
     </row>
   </sheetData>

</xml_diff>